<commit_message>
Added event icons; fixed minor issues
Added custom SVGs for event subtypes "strike," "disease," and "nature."
Removed low opacity markers for entries that are not within the selected year in the temporal filter.
Fixed date errors in nodes.csv.
</commit_message>
<xml_diff>
--- a/data/nodes.xlsx
+++ b/data/nodes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro\Documents\GitHub\in-the-shadow-of-the-banana\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D90F11B7-E01B-46F1-81D6-2EB71D74DA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{898A7DEF-CEA7-4DDA-8242-D4FDCD679C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5B9B3091-99AB-4305-BC97-7032E7BEE02C}"/>
   </bookViews>
@@ -2384,6 +2384,12 @@
       <c r="F26" t="b">
         <v>1</v>
       </c>
+      <c r="H26">
+        <v>1934</v>
+      </c>
+      <c r="I26">
+        <v>1934</v>
+      </c>
       <c r="J26" t="b">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Legend Panel Change and Minor Fixes
* Removed legend from "Search/Filter" bar and created its own separate panel on the left; organized legend by type; enlarged legend icons.
* Changed "event" relational type to "action," to distinguish it from the "event" entry type.
* Added custom icon for port entry markers.
* Added new event subtypes "mediation" and "exploitation."
* Added new entry type "migration" and subtype "displacement."
* Changed UFCo-related entry colors to a cohesive set of whites and grays.
* Made side panel sticky so that the close button doesn't disappear when scrolling down.
</commit_message>
<xml_diff>
--- a/data/nodes.xlsx
+++ b/data/nodes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro\Documents\GitHub\in-the-shadow-of-the-banana\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{898A7DEF-CEA7-4DDA-8242-D4FDCD679C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695D6108-7C04-4E0F-A8B2-9BFB98B50C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5B9B3091-99AB-4305-BC97-7032E7BEE02C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="293">
   <si>
     <t>id</t>
   </si>
@@ -996,21 +996,9 @@
     <t>Declaration of Strike</t>
   </si>
   <si>
-    <t>1934_strike_marker_001</t>
-  </si>
-  <si>
-    <t>1934_strike_marker_002</t>
-  </si>
-  <si>
     <t>1934_strike_marker_003</t>
   </si>
   <si>
-    <t>1934_strike_marker_004</t>
-  </si>
-  <si>
-    <t>1934_strike_marker_005</t>
-  </si>
-  <si>
     <t>worker_meeting_01_1934</t>
   </si>
   <si>
@@ -1057,6 +1045,15 @@
   </si>
   <si>
     <t>Cuartel general de los huelguistas durante la huelga bananera de 1934.</t>
+  </si>
+  <si>
+    <t>action</t>
+  </si>
+  <si>
+    <t>exploitation</t>
+  </si>
+  <si>
+    <t>public_site</t>
   </si>
 </sst>
 </file>
@@ -1112,12 +1109,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1136,8 +1130,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8DE4AF77-3078-41E5-A862-A672CD070CDC}" name="Table2" displayName="Table2" ref="A1:Y70" totalsRowShown="0">
-  <autoFilter ref="A1:Y70" xr:uid="{8DE4AF77-3078-41E5-A862-A672CD070CDC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8DE4AF77-3078-41E5-A862-A672CD070CDC}" name="Table2" displayName="Table2" ref="A1:Y66" totalsRowShown="0">
+  <autoFilter ref="A1:Y66" xr:uid="{8DE4AF77-3078-41E5-A862-A672CD070CDC}"/>
   <tableColumns count="25">
     <tableColumn id="1" xr3:uid="{BA8A667B-2EA1-408D-ABAE-261F71369134}" name="id"/>
     <tableColumn id="2" xr3:uid="{1E8557DA-5346-4170-9098-68F69CB64A7F}" name="label_en"/>
@@ -1486,7 +1480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21EAC64A-5CB7-4B0B-817E-D41EE9B9A394}">
-  <dimension ref="A1:Y70"/>
+  <dimension ref="A1:Y66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
@@ -2083,7 +2077,7 @@
         <v>152</v>
       </c>
       <c r="U16" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="X16" t="s">
         <v>114</v>
@@ -2924,7 +2918,7 @@
         <v>257</v>
       </c>
       <c r="D45" t="s">
-        <v>72</v>
+        <v>290</v>
       </c>
       <c r="E45" t="s">
         <v>106</v>
@@ -3206,6 +3200,9 @@
       <c r="D50" t="s">
         <v>72</v>
       </c>
+      <c r="E50" t="s">
+        <v>291</v>
+      </c>
       <c r="F50" t="s">
         <v>136</v>
       </c>
@@ -3220,6 +3217,12 @@
       </c>
       <c r="J50" t="b">
         <v>1</v>
+      </c>
+      <c r="K50" s="1">
+        <v>-83.033799999999999</v>
+      </c>
+      <c r="L50" s="1">
+        <v>9.9901999999999997</v>
       </c>
       <c r="M50" t="s">
         <v>165</v>
@@ -3239,10 +3242,10 @@
         <v>260</v>
       </c>
       <c r="B51" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="C51" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D51" t="s">
         <v>168</v>
@@ -3301,7 +3304,7 @@
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="B52" t="s">
         <v>262</v>
@@ -3343,10 +3346,10 @@
         <v>1</v>
       </c>
       <c r="T52" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="U52" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="X52" t="s">
         <v>114</v>
@@ -3363,7 +3366,7 @@
         <v>272</v>
       </c>
       <c r="C53" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="D53" t="s">
         <v>168</v>
@@ -3396,16 +3399,16 @@
         <v>17</v>
       </c>
       <c r="T53" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="U53" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="X53" t="s">
         <v>114</v>
       </c>
       <c r="Y53" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.25">
@@ -3413,10 +3416,10 @@
         <v>273</v>
       </c>
       <c r="B54" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="C54" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="D54" t="s">
         <v>72</v>
@@ -3440,16 +3443,19 @@
         <v>1</v>
       </c>
       <c r="K54">
-        <v>-83.299000000000007</v>
+        <v>-83.355490700000004</v>
       </c>
       <c r="L54">
-        <v>10.065</v>
+        <v>10.0877643</v>
+      </c>
+      <c r="M54" t="s">
+        <v>165</v>
       </c>
       <c r="T54" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="U54" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="X54" t="s">
         <v>114</v>
@@ -3460,25 +3466,25 @@
     </row>
     <row r="55" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>274</v>
+        <v>118</v>
       </c>
       <c r="B55" t="s">
-        <v>280</v>
+        <v>223</v>
       </c>
       <c r="C55" t="s">
-        <v>281</v>
+        <v>146</v>
       </c>
       <c r="D55" t="s">
-        <v>72</v>
+        <v>290</v>
       </c>
       <c r="E55" t="s">
-        <v>73</v>
+        <v>106</v>
       </c>
       <c r="F55" t="s">
         <v>136</v>
       </c>
       <c r="G55">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H55">
         <v>1934</v>
@@ -3487,19 +3493,31 @@
         <v>1934</v>
       </c>
       <c r="J55" t="b">
-        <v>1</v>
-      </c>
-      <c r="K55">
-        <v>-83.05</v>
-      </c>
-      <c r="L55">
-        <v>10</v>
+        <v>0</v>
+      </c>
+      <c r="M55" t="s">
+        <v>165</v>
+      </c>
+      <c r="N55" t="s">
+        <v>119</v>
+      </c>
+      <c r="O55" t="s">
+        <v>27</v>
+      </c>
+      <c r="P55" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>93</v>
+      </c>
+      <c r="R55" t="s">
+        <v>117</v>
       </c>
       <c r="T55" t="s">
-        <v>283</v>
+        <v>162</v>
       </c>
       <c r="U55" t="s">
-        <v>284</v>
+        <v>161</v>
       </c>
       <c r="X55" t="s">
         <v>114</v>
@@ -3510,25 +3528,25 @@
     </row>
     <row r="56" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>275</v>
+        <v>119</v>
       </c>
       <c r="B56" t="s">
-        <v>280</v>
+        <v>222</v>
       </c>
       <c r="C56" t="s">
-        <v>281</v>
+        <v>145</v>
       </c>
       <c r="D56" t="s">
-        <v>72</v>
+        <v>290</v>
       </c>
       <c r="E56" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="F56" t="s">
         <v>136</v>
       </c>
       <c r="G56">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H56">
         <v>1934</v>
@@ -3539,17 +3557,29 @@
       <c r="J56" t="b">
         <v>1</v>
       </c>
-      <c r="K56">
-        <v>-82.957999999999998</v>
-      </c>
-      <c r="L56" s="2">
-        <v>9.9779999999999998</v>
+      <c r="K56" s="1">
+        <v>-83.54</v>
+      </c>
+      <c r="L56" s="1">
+        <v>10.1</v>
+      </c>
+      <c r="M56" t="s">
+        <v>165</v>
+      </c>
+      <c r="P56" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>107</v>
+      </c>
+      <c r="R56" t="s">
+        <v>136</v>
       </c>
       <c r="T56" t="s">
-        <v>283</v>
+        <v>211</v>
       </c>
       <c r="U56" t="s">
-        <v>284</v>
+        <v>163</v>
       </c>
       <c r="X56" t="s">
         <v>114</v>
@@ -3560,25 +3590,25 @@
     </row>
     <row r="57" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>276</v>
+        <v>186</v>
       </c>
       <c r="B57" t="s">
-        <v>280</v>
+        <v>221</v>
       </c>
       <c r="C57" t="s">
-        <v>281</v>
+        <v>188</v>
       </c>
       <c r="D57" t="s">
-        <v>72</v>
+        <v>290</v>
       </c>
       <c r="E57" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="F57" t="s">
         <v>136</v>
       </c>
       <c r="G57">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H57">
         <v>1934</v>
@@ -3587,19 +3617,31 @@
         <v>1934</v>
       </c>
       <c r="J57" t="b">
-        <v>1</v>
-      </c>
-      <c r="K57">
-        <v>-83.12</v>
-      </c>
-      <c r="L57">
-        <v>9.98</v>
+        <v>0</v>
+      </c>
+      <c r="M57" t="s">
+        <v>165</v>
+      </c>
+      <c r="N57" t="s">
+        <v>18</v>
+      </c>
+      <c r="O57" t="s">
+        <v>48</v>
+      </c>
+      <c r="P57" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>107</v>
+      </c>
+      <c r="R57" t="s">
+        <v>136</v>
       </c>
       <c r="T57" t="s">
-        <v>283</v>
+        <v>190</v>
       </c>
       <c r="U57" t="s">
-        <v>284</v>
+        <v>189</v>
       </c>
       <c r="X57" t="s">
         <v>114</v>
@@ -3610,25 +3652,25 @@
     </row>
     <row r="58" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>277</v>
+        <v>187</v>
       </c>
       <c r="B58" t="s">
-        <v>280</v>
+        <v>220</v>
       </c>
       <c r="C58" t="s">
-        <v>281</v>
+        <v>192</v>
       </c>
       <c r="D58" t="s">
-        <v>72</v>
+        <v>290</v>
       </c>
       <c r="E58" t="s">
-        <v>73</v>
+        <v>191</v>
       </c>
       <c r="F58" t="s">
         <v>136</v>
       </c>
       <c r="G58">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H58">
         <v>1934</v>
@@ -3637,19 +3679,31 @@
         <v>1934</v>
       </c>
       <c r="J58" t="b">
-        <v>1</v>
-      </c>
-      <c r="K58">
-        <v>-82.620999999999995</v>
-      </c>
-      <c r="L58">
-        <v>9.5269999999999992</v>
+        <v>0</v>
+      </c>
+      <c r="M58" t="s">
+        <v>165</v>
+      </c>
+      <c r="N58" t="s">
+        <v>48</v>
+      </c>
+      <c r="O58" t="s">
+        <v>18</v>
+      </c>
+      <c r="P58" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>136</v>
+      </c>
+      <c r="R58" t="s">
+        <v>107</v>
       </c>
       <c r="T58" t="s">
-        <v>283</v>
+        <v>209</v>
       </c>
       <c r="U58" t="s">
-        <v>284</v>
+        <v>208</v>
       </c>
       <c r="X58" t="s">
         <v>114</v>
@@ -3660,16 +3714,16 @@
     </row>
     <row r="59" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>118</v>
+        <v>219</v>
       </c>
       <c r="B59" t="s">
-        <v>223</v>
+        <v>285</v>
       </c>
       <c r="C59" t="s">
-        <v>146</v>
+        <v>286</v>
       </c>
       <c r="D59" t="s">
-        <v>72</v>
+        <v>290</v>
       </c>
       <c r="E59" t="s">
         <v>106</v>
@@ -3678,7 +3732,7 @@
         <v>136</v>
       </c>
       <c r="G59">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H59">
         <v>1934</v>
@@ -3693,116 +3747,89 @@
         <v>165</v>
       </c>
       <c r="N59" t="s">
-        <v>119</v>
+        <v>48</v>
       </c>
       <c r="O59" t="s">
-        <v>27</v>
+        <v>210</v>
       </c>
       <c r="P59" t="b">
         <v>1</v>
       </c>
-      <c r="Q59" t="s">
-        <v>93</v>
-      </c>
-      <c r="R59" t="s">
-        <v>117</v>
-      </c>
       <c r="T59" t="s">
-        <v>162</v>
+        <v>218</v>
       </c>
       <c r="U59" t="s">
-        <v>161</v>
+        <v>217</v>
       </c>
       <c r="X59" t="s">
         <v>114</v>
       </c>
       <c r="Y59">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="60" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>119</v>
+        <v>210</v>
       </c>
       <c r="B60" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="C60" t="s">
-        <v>145</v>
+        <v>213</v>
       </c>
       <c r="D60" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="E60" t="s">
-        <v>108</v>
-      </c>
-      <c r="F60" t="s">
-        <v>136</v>
-      </c>
-      <c r="G60">
-        <v>8</v>
+        <v>292</v>
       </c>
       <c r="H60">
-        <v>1934</v>
+        <v>1855</v>
       </c>
       <c r="I60">
-        <v>1934</v>
+        <v>1958</v>
       </c>
       <c r="J60" t="b">
         <v>1</v>
       </c>
-      <c r="K60" s="1">
-        <v>-83.54</v>
-      </c>
-      <c r="L60" s="1">
-        <v>10.1</v>
+      <c r="K60">
+        <v>-84.085564000000005</v>
+      </c>
+      <c r="L60">
+        <v>9.9354469999999999</v>
       </c>
       <c r="M60" t="s">
         <v>165</v>
       </c>
-      <c r="P60" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q60" t="s">
-        <v>107</v>
-      </c>
-      <c r="R60" t="s">
-        <v>136</v>
-      </c>
       <c r="T60" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="U60" t="s">
-        <v>163</v>
-      </c>
-      <c r="X60" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y60">
-        <v>88</v>
+        <v>225</v>
       </c>
     </row>
     <row r="61" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>186</v>
+        <v>212</v>
       </c>
       <c r="B61" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="C61" t="s">
-        <v>188</v>
+        <v>227</v>
       </c>
       <c r="D61" t="s">
         <v>72</v>
       </c>
       <c r="E61" t="s">
-        <v>108</v>
+        <v>224</v>
       </c>
       <c r="F61" t="s">
         <v>136</v>
       </c>
       <c r="G61">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H61">
         <v>1934</v>
@@ -3811,60 +3838,51 @@
         <v>1934</v>
       </c>
       <c r="J61" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K61">
+        <v>-84.085564000000005</v>
+      </c>
+      <c r="L61">
+        <v>9.9354469999999999</v>
       </c>
       <c r="M61" t="s">
         <v>165</v>
       </c>
-      <c r="N61" t="s">
-        <v>18</v>
-      </c>
-      <c r="O61" t="s">
-        <v>48</v>
-      </c>
-      <c r="P61" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q61" t="s">
-        <v>107</v>
-      </c>
-      <c r="R61" t="s">
-        <v>136</v>
-      </c>
       <c r="T61" t="s">
-        <v>190</v>
+        <v>215</v>
       </c>
       <c r="U61" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="X61" t="s">
         <v>114</v>
       </c>
       <c r="Y61">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="62" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>187</v>
+        <v>228</v>
       </c>
       <c r="B62" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="C62" t="s">
-        <v>192</v>
+        <v>230</v>
       </c>
       <c r="D62" t="s">
-        <v>72</v>
+        <v>290</v>
       </c>
       <c r="E62" t="s">
-        <v>191</v>
+        <v>106</v>
       </c>
       <c r="F62" t="s">
         <v>136</v>
       </c>
       <c r="G62">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H62">
         <v>1934</v>
@@ -3879,54 +3897,48 @@
         <v>165</v>
       </c>
       <c r="N62" t="s">
+        <v>210</v>
+      </c>
+      <c r="O62" t="s">
         <v>48</v>
       </c>
-      <c r="O62" t="s">
-        <v>18</v>
-      </c>
       <c r="P62" t="b">
         <v>1</v>
       </c>
-      <c r="Q62" t="s">
-        <v>136</v>
-      </c>
-      <c r="R62" t="s">
-        <v>107</v>
-      </c>
       <c r="T62" t="s">
-        <v>209</v>
+        <v>231</v>
       </c>
       <c r="U62" t="s">
-        <v>208</v>
+        <v>232</v>
       </c>
       <c r="X62" t="s">
         <v>114</v>
       </c>
       <c r="Y62">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="63" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="B63" t="s">
-        <v>289</v>
+        <v>234</v>
       </c>
       <c r="C63" t="s">
+        <v>235</v>
+      </c>
+      <c r="D63" t="s">
         <v>290</v>
       </c>
-      <c r="D63" t="s">
-        <v>72</v>
-      </c>
       <c r="E63" t="s">
-        <v>106</v>
+        <v>191</v>
       </c>
       <c r="F63" t="s">
         <v>136</v>
       </c>
       <c r="G63">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H63">
         <v>1934</v>
@@ -3940,330 +3952,124 @@
       <c r="M63" t="s">
         <v>165</v>
       </c>
-      <c r="N63" t="s">
-        <v>48</v>
-      </c>
-      <c r="O63" t="s">
-        <v>210</v>
-      </c>
-      <c r="P63" t="b">
-        <v>1</v>
-      </c>
       <c r="T63" t="s">
-        <v>218</v>
+        <v>236</v>
       </c>
       <c r="U63" t="s">
-        <v>217</v>
+        <v>237</v>
       </c>
       <c r="X63" t="s">
         <v>114</v>
       </c>
       <c r="Y63">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="64" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="B64" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="C64" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="D64" t="s">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="E64" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="H64">
-        <v>1855</v>
+        <v>1928</v>
       </c>
       <c r="I64">
-        <v>1958</v>
+        <v>1928</v>
       </c>
       <c r="J64" t="b">
         <v>1</v>
       </c>
       <c r="K64">
-        <v>-84.085564000000005</v>
+        <v>-74.247649999999993</v>
       </c>
       <c r="L64">
-        <v>9.9354469999999999</v>
+        <v>11.00703</v>
       </c>
       <c r="M64" t="s">
-        <v>165</v>
+        <v>199</v>
       </c>
       <c r="T64" t="s">
-        <v>214</v>
-      </c>
-      <c r="U64" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="65" spans="1:25" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="B65" t="s">
-        <v>226</v>
+        <v>202</v>
       </c>
       <c r="C65" t="s">
-        <v>227</v>
+        <v>205</v>
       </c>
       <c r="D65" t="s">
         <v>72</v>
       </c>
       <c r="E65" t="s">
-        <v>224</v>
-      </c>
-      <c r="F65" t="s">
-        <v>136</v>
-      </c>
-      <c r="G65">
-        <v>12</v>
+        <v>73</v>
       </c>
       <c r="H65">
-        <v>1934</v>
+        <v>1960</v>
       </c>
       <c r="I65">
-        <v>1934</v>
+        <v>1960</v>
       </c>
       <c r="J65" t="b">
         <v>1</v>
       </c>
       <c r="K65">
-        <v>-84.085564000000005</v>
+        <v>-79.680000000000007</v>
       </c>
       <c r="L65">
-        <v>9.9354469999999999</v>
+        <v>9.08</v>
       </c>
       <c r="M65" t="s">
-        <v>165</v>
-      </c>
-      <c r="T65" t="s">
-        <v>215</v>
-      </c>
-      <c r="U65" t="s">
-        <v>216</v>
-      </c>
-      <c r="X65" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y65">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="66" spans="1:25" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>228</v>
+        <v>204</v>
       </c>
       <c r="B66" t="s">
-        <v>229</v>
+        <v>203</v>
       </c>
       <c r="C66" t="s">
-        <v>230</v>
+        <v>206</v>
       </c>
       <c r="D66" t="s">
         <v>72</v>
       </c>
       <c r="E66" t="s">
-        <v>224</v>
-      </c>
-      <c r="F66" t="s">
-        <v>136</v>
-      </c>
-      <c r="G66">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="H66">
-        <v>1934</v>
+        <v>1964</v>
       </c>
       <c r="I66">
-        <v>1934</v>
+        <v>1964</v>
       </c>
       <c r="J66" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K66">
+        <v>-82.86206</v>
+      </c>
+      <c r="L66">
+        <v>8.2777499999999993</v>
       </c>
       <c r="M66" t="s">
-        <v>165</v>
-      </c>
-      <c r="N66" t="s">
-        <v>210</v>
-      </c>
-      <c r="O66" t="s">
-        <v>48</v>
-      </c>
-      <c r="P66" t="b">
-        <v>1</v>
-      </c>
-      <c r="T66" t="s">
-        <v>231</v>
-      </c>
-      <c r="U66" t="s">
-        <v>232</v>
-      </c>
-      <c r="X66" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y66">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="67" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>233</v>
-      </c>
-      <c r="B67" t="s">
-        <v>234</v>
-      </c>
-      <c r="C67" t="s">
-        <v>235</v>
-      </c>
-      <c r="D67" t="s">
-        <v>72</v>
-      </c>
-      <c r="E67" t="s">
-        <v>191</v>
-      </c>
-      <c r="F67" t="s">
-        <v>136</v>
-      </c>
-      <c r="G67">
-        <v>14</v>
-      </c>
-      <c r="H67">
-        <v>1934</v>
-      </c>
-      <c r="I67">
-        <v>1934</v>
-      </c>
-      <c r="J67" t="b">
-        <v>0</v>
-      </c>
-      <c r="M67" t="s">
-        <v>165</v>
-      </c>
-      <c r="T67" t="s">
-        <v>236</v>
-      </c>
-      <c r="U67" t="s">
-        <v>237</v>
-      </c>
-      <c r="X67" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y67">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="68" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>196</v>
-      </c>
-      <c r="B68" t="s">
-        <v>197</v>
-      </c>
-      <c r="C68" t="s">
-        <v>198</v>
-      </c>
-      <c r="D68" t="s">
-        <v>72</v>
-      </c>
-      <c r="E68" t="s">
-        <v>73</v>
-      </c>
-      <c r="H68">
-        <v>1928</v>
-      </c>
-      <c r="I68">
-        <v>1928</v>
-      </c>
-      <c r="J68" t="b">
-        <v>1</v>
-      </c>
-      <c r="K68">
-        <v>-74.247649999999993</v>
-      </c>
-      <c r="L68">
-        <v>11.00703</v>
-      </c>
-      <c r="M68" t="s">
-        <v>199</v>
-      </c>
-      <c r="T68" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="69" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>201</v>
-      </c>
-      <c r="B69" t="s">
-        <v>202</v>
-      </c>
-      <c r="C69" t="s">
-        <v>205</v>
-      </c>
-      <c r="D69" t="s">
-        <v>72</v>
-      </c>
-      <c r="E69" t="s">
-        <v>73</v>
-      </c>
-      <c r="H69">
-        <v>1960</v>
-      </c>
-      <c r="I69">
-        <v>1960</v>
-      </c>
-      <c r="J69" t="b">
-        <v>1</v>
-      </c>
-      <c r="K69">
-        <v>-79.680000000000007</v>
-      </c>
-      <c r="L69">
-        <v>9.08</v>
-      </c>
-      <c r="M69" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="70" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>204</v>
-      </c>
-      <c r="B70" t="s">
-        <v>203</v>
-      </c>
-      <c r="C70" t="s">
-        <v>206</v>
-      </c>
-      <c r="D70" t="s">
-        <v>72</v>
-      </c>
-      <c r="E70" t="s">
-        <v>73</v>
-      </c>
-      <c r="H70">
-        <v>1964</v>
-      </c>
-      <c r="I70">
-        <v>1964</v>
-      </c>
-      <c r="J70" t="b">
-        <v>1</v>
-      </c>
-      <c r="K70">
-        <v>-82.86206</v>
-      </c>
-      <c r="L70">
-        <v>8.2777499999999993</v>
-      </c>
-      <c r="M70" t="s">
         <v>207</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added/fixed data, improved user interface, and fixed bezier curve alternance and offset in sequence animations.
* Updated sequence.js popups to display more entry information (type, title, date, description, and source).
* Updated parent_event.html to no longer displays connections, as they were redundant with the sequence.
* Updated render.py to use translations.js instead of translations.json, as they were redundant.
* Updated legend button so '≡' is replaced with 'x' when the legend panel is open.
* Fixed issue in sequence.js: Bezier curve indexes now carry over to later events so that curves between the same locations don't fully overlap.
* Updated nodes.csv: Improved writing, fixed typos, and reclassified some events as different relation types. Extended the "1934 Banana Strike" sequence with more events based on Cerdas (1984).
* Added "deportation" as a migration subtype.
* Added "conflict" as an event subtype.
</commit_message>
<xml_diff>
--- a/data/nodes.xlsx
+++ b/data/nodes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro\Documents\GitHub\in-the-shadow-of-the-banana\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695D6108-7C04-4E0F-A8B2-9BFB98B50C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAEAA03-7BB0-45A6-A947-31A99F32C5A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5B9B3091-99AB-4305-BC97-7032E7BEE02C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="320">
   <si>
     <t>id</t>
   </si>
@@ -428,9 +428,6 @@
     <t>Ferrocarril al Pacífico</t>
   </si>
   <si>
-    <t>la_fortuna</t>
-  </si>
-  <si>
     <t>la_perla</t>
   </si>
   <si>
@@ -455,9 +452,6 @@
     <t>Banana Strike of 1934</t>
   </si>
   <si>
-    <t>Huelga Bananera de 1934</t>
-  </si>
-  <si>
     <t>FFCC Internacionales de Centro America</t>
   </si>
   <si>
@@ -530,9 +524,6 @@
     <t>Manuel Mora relies on his congressional immunity to avoid arrest and invoke habeas corpus in the Siquirres court to release workers arrested during the Banana Strike of 1934.</t>
   </si>
   <si>
-    <t>Para detener la huelga de 1934, el Gobierno de Costa Rica ordena a la Fuerza Pública detener a los huelguistas que transiten por los caminos públicos.</t>
-  </si>
-  <si>
     <t>country</t>
   </si>
   <si>
@@ -608,15 +599,6 @@
     <t>La Fuerza Pública corta y recoge el banano</t>
   </si>
   <si>
-    <t>La Fuerza Pública es enviada a cortar y recoger banano para reemplazar a los huelguistas y contener la huega.</t>
-  </si>
-  <si>
-    <t>Police forces are sent to cut and collect bananas to replace the workers and contain the strike.</t>
-  </si>
-  <si>
-    <t>violence</t>
-  </si>
-  <si>
     <t>Obreros destruyen banano</t>
   </si>
   <si>
@@ -665,16 +647,7 @@
     <t>Panama</t>
   </si>
   <si>
-    <t>Los huelguistas responden destruyendo 10 hectáreas de banano en la noche, evitando que llegue banano bueno a Limón.</t>
-  </si>
-  <si>
-    <t>Workers respond by destroying 10 hectares of bananas at  night, preventing any good bananas from reaching Limón.</t>
-  </si>
-  <si>
     <t>palacio_nacional</t>
-  </si>
-  <si>
-    <t>To stop the strike of 1934, the mayor orders the police to arrest striking workers as they transit public roads.</t>
   </si>
   <si>
     <t>jimenez_meetings_1934</t>
@@ -731,32 +704,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">The Executive Power, headed by President Ricardo Jiménez Oreamuno, convened a series of consultative meetings at the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>National Palace</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> to mediate the 1934 banana strike. During these sessions, the Presidency interrogated key stakeholders, including plantation owner Arturo Volio. Upon Volio’s admission of the prevailing labor conditions, the Executive formally attributed responsibility for the industrial action to the banana companies’ management practices.</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">El Poder Ejecutivo, encabezado por el presidente Ricardo Jiménez Oreamuno, convocó una serie de reuniones consultivas en el </t>
     </r>
     <r>
@@ -868,192 +815,326 @@
     <t>Inspección ministerial en 26 Millas</t>
   </si>
   <si>
+    <t>Countermanded Order of Sabotage</t>
+  </si>
+  <si>
+    <t>Contraorden de sabotaje</t>
+  </si>
+  <si>
+    <t>During a period of heightened tension in the 1934 strike, Carlos Luis Fallas—acting on unverified intelligence regarding approaching authorities—issued a written order to destroy a bridge to impede troop movement. Jaime Cerdas, co-leader of the movement, disputed the decision and unilaterally issued a countermand, nullifying the sabotage order without Fallas's immediate knowledge.</t>
+  </si>
+  <si>
+    <t>Durante un periodo de alta tensión en la huelga de 1934, Carlos Luis Fallas—actuando bajo inteligencia no verificada sobre el avance de las autoridades—emitió una orden escrita para destruir un puente y así impedir el movimiento de tropas. Jaime Cerdas, codirigente del movimiento, cuestionó la decisión y emitió unilateralmente una contraorden, anulando el sabotaje sin el conocimiento inmediato de Fallas.</t>
+  </si>
+  <si>
+    <t>Malaria Outbreak: Guápiles Sector</t>
+  </si>
+  <si>
+    <t>Brote de malaria: Sector Guápiles</t>
+  </si>
+  <si>
+    <t>migration</t>
+  </si>
+  <si>
+    <t>displacement</t>
+  </si>
+  <si>
+    <t>Sanitary Displacement: Guápiles to Siquirres</t>
+  </si>
+  <si>
+    <t>Desplazamiento sanitario: De Guápiles a Siquirres</t>
+  </si>
+  <si>
+    <t>Malaria Outbreak: Remote Plantations</t>
+  </si>
+  <si>
+    <t>Brote de malaria: Fincas remotas</t>
+  </si>
+  <si>
+    <t>Desplazamiento sanitario: Fincas remotas a Limón</t>
+  </si>
+  <si>
+    <t>Sanitary Displacement: Remote Plantations to Limón</t>
+  </si>
+  <si>
+    <t>Jaime Cerdas Mora reports a lack of medical infrastructure in the Guápiles sector. He notes that there were no resident doctors or local hospitals, leaving workers without immediate care during malaria outbreaks.</t>
+  </si>
+  <si>
+    <t>Jaime Cerdas Mora informa sobre la falta de infraestructura médica en el sector de Guápiles. Señala que no había médicos residentes ni hospitales locales, lo que dejaba a los trabajadores sin atención inmediata durante los brotes de malaria.</t>
+  </si>
+  <si>
+    <t>Jaime Cerdas Mora states that in remote plantations, malaria cases were frequent due to workers living in flooded barracks (ranchones). He estimates that half of the workers were unable to work half of the time because of the disease.</t>
+  </si>
+  <si>
+    <t>Jaime Cerdas Mora afirma que en fincas remotas, los casos de malaria eran frecuentes debido a que los trabajadores vivían en barracones (ranchones) inundados. Estima que la mitad de los trabajadores no podía laborar la mitad del tiempo a causa de la enfermedad.</t>
+  </si>
+  <si>
+    <t>Cerdas describes workers from Guápiles traveling to Siquirres for treatment. He identifies the facility there as a dispensary staffed by a nurse rather than a doctor, where quinine was the only medicine provided.</t>
+  </si>
+  <si>
+    <t>Cerdas describe a los trabajadores de Guápiles viajando a Siquirres para recibir tratamiento. Identifica la instalación allí como un dispensario atendido por un enfermero en lugar de un médico, donde la quinina era el único medicamento suministrado.</t>
+  </si>
+  <si>
+    <t>Cerdas explains that workers in remote areas, such as those near the Sixaola river, were forced to travel to the city of Limón to find a hospital. This required sick laborers to travel long distances from the plantations to the provincial capital.</t>
+  </si>
+  <si>
+    <t>Cerdas explica que los trabajadores de zonas remotas, como las cercanas al río Sixaola, se veían obligados a trasladarse a la ciudad de Limón para encontrar un hospital. Esto requería que los obreros enfermos viajaran largas distancias desde las fincas hasta la capital provincial.</t>
+  </si>
+  <si>
+    <t>Judicial Confinement of Carlos Luis Fallas to Limón</t>
+  </si>
+  <si>
+    <t>Confinamiento judicial de Carlos Luis Fallas a Limón</t>
+  </si>
+  <si>
+    <t>declaration_strike_1934</t>
+  </si>
+  <si>
+    <t>demands_strike_1934</t>
+  </si>
+  <si>
+    <t>Según el relato de Jaime Cerdas Mora, el Partido Comunista redactó un pliego de peticiones formal y organizó comités de huelga en las diversas fincas bananeras. El documento fue presentado al gerente de la United Fruit Company, George P. Chittenden, quien se negó a recibirlo.</t>
+  </si>
+  <si>
+    <t>Leadership Deployment to 26 Millas</t>
+  </si>
+  <si>
+    <t>Despliegue de la dirigencia hacia 26 Millas</t>
+  </si>
+  <si>
+    <t>movement</t>
+  </si>
+  <si>
+    <t>comisariatos_1934_strike</t>
+  </si>
+  <si>
+    <t>Los comisariatos vinculados a la UFCo y a las fincas bananeras formaban un sistema de dependencia económica a lo largo de la zona bananera atlántica. Con frecuencia, los trabajadores eran pagados mediante cupones o chapas que solo podían utilizarse en los comisariatos de las plantaciones, donde los productos se vendían a precios elevados. Según el relato de Jaime Cerdas, este sistema agravaba los bajos salarios y las malas condiciones de vida, produciendo una “doble explotación” de los trabajadores bananeros a través tanto del trabajo como del consumo controlado.</t>
+  </si>
+  <si>
+    <t>Declaration of Strike</t>
+  </si>
+  <si>
+    <t>1934_strike_marker_003</t>
+  </si>
+  <si>
+    <t>worker_meeting_01_1934</t>
+  </si>
+  <si>
+    <t>87–88</t>
+  </si>
+  <si>
+    <t>Paralysis of the Atlantic Region</t>
+  </si>
+  <si>
+    <t>La paralización de la zona atlántica</t>
+  </si>
+  <si>
+    <t>Declaración de la huelga</t>
+  </si>
+  <si>
+    <t>By the day following its formal declaration, the 1934 banana strike had spread across the Atlantic banana zone. According to Jaime Cerdas, plantations throughout the region had already joined the movement, paralyzing production, transportation, and UFCo operations across the corridor.</t>
+  </si>
+  <si>
+    <t>Para el día siguiente de su declaración formal, la huelga bananera de 1934 ya se había extendido por toda la zona bananera atlántica. Según Jaime Cerdas, plantaciones a lo largo de la región se habían incorporado al movimiento, paralizando la producción, el transporte y las operaciones de la UFCo en todo el corredor bananero.</t>
+  </si>
+  <si>
+    <t>Tras el rechazo del pliego de peticiones de los trabajadores por parte del gerente de la UFCo, George P. Chittenden. Los obreros sostuvieron una reunión cerca del 7 de agosto de 1934, en la que se acordó ir a huelga. Para entonces, ya se habían organizado comités de huelga en múltiples plantaciones, y Carlos Luis Fallas y Jaime Cerdas fueron encargados de dirigir el movimiento. Viajando en tren hasta Madre de Dios y luego a pie hacia 26 Millas, establecieron el principal cuartel operativo de la huelga cerca de la finca Los Ángeles. Según el relato de Cerdas, delegaciones de plantaciones a lo largo del corredor bananero atlántico ya se estaban reuniendo allí al momento de su llegada.</t>
+  </si>
+  <si>
+    <t>On August 9, 1934, strike leaders formally declared the beginning of the banana strike. The declaration marked the transition from localized labor grievances to a coordinated regional movement across the Atlantic banana zone.</t>
+  </si>
+  <si>
+    <t>El 9 de agosto de 1934, los dirigentes huelguistas declararon formalmente el inicio de la huelga bananera. La declaración marcó la transición de reclamos laborales localizados hacia un movimiento coordinado a escala regional en la zona bananera atlántica.</t>
+  </si>
+  <si>
+    <t>Deposition of Carlos Luis Fallas</t>
+  </si>
+  <si>
+    <t>Deposición de Carlos Luis Fallas</t>
+  </si>
+  <si>
+    <t>Presentación y rechazo del pliego de peticiones</t>
+  </si>
+  <si>
+    <t>Presentation and Rejection of the List of Demands</t>
+  </si>
+  <si>
+    <t>Cuartel general de los huelguistas durante la huelga bananera de 1934.</t>
+  </si>
+  <si>
+    <t>action</t>
+  </si>
+  <si>
+    <t>exploitation</t>
+  </si>
+  <si>
+    <t>public_site</t>
+  </si>
+  <si>
+    <t>deportation</t>
+  </si>
+  <si>
+    <t>Commissaries and the Scrip System</t>
+  </si>
+  <si>
+    <t>Los comisariatos y los cupones de la compañía</t>
+  </si>
+  <si>
+    <t>UFCo and plantation-linked commissaries formed a system of economic dependency across the Atlantic banana zone. Workers were frequently paid with coupons or tokens redeemable only at plantation commissaries, where goods were sold at inflated prices. According to Jaime Cerdas, this arrangement compounded already poor wages and living conditions, reinforcing what he described as a “double exploitation” of banana workers through both labor and controlled consumption.</t>
+  </si>
+  <si>
+    <t>Following a strike organized in Alajuela, judicial authorities sentenced Carlos Luis Fallas to confinement in Limón, where he arrives in December 1933. This was a common legal penalty at the time, used to isolate political and labor leaders from their active organizational bases.</t>
+  </si>
+  <si>
+    <t>Tras una huelga que organizó en Alajuela, las autoridades judiciales sentenciaron a Carlos Luis Fallas a la pena de confinamiento en Limón, adonde llega en diciembre de 1933. Esta era una sanción legal común en la época, utilizada para aislar a líderes políticos y sindicales de sus bases organizativas activas.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The Executive Power, headed by President Ricardo Jiménez Oreamuno, convened a series of consultative meetings at the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>National Palace</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to mediate the 1934 banana strike. During these sessions, the Presidency interrogated key stakeholders, including plantation owner Arturo Volio. Upon Volio’s admission of the prevailing labor conditions, the Executive formally attributed responsibility for the conflict to the banana industry's management practices.</t>
+    </r>
+  </si>
+  <si>
     <t>The Minister of Government and Labor, Santos León Herrera, accompanied by the Chief of the Labor Section, Zayas Bazán, conducted a field inspection at the 26 Millas plantation during the absence of Carlos Luis Fallas. The visit functioned as a direct observation of the living quarters (ranchones), where the delegation encountered flooded dwellings and active cases of malaria.
-The event is noted for its impact on the Minister’s legislative perspective. After witnessing the conditions and the confinement of workers, León Herrera explicitly conceded a divergence between "legality" and "justice."</t>
+The event is noted for its impact on the Minister’s perspective. After witnessing the conditions and the confinement of workers, León Herrera explicitly conceded a divergence between "legality" and "justice."</t>
   </si>
   <si>
     <t>El Ministro de Gobernación y Trabajo, Santos León Herrera, acompañado por el Jefe de la Sección de Trabajo, Zayas Bazán, realizó una inspección de campo en la finca 26 Millas durante la ausencia de Carlos Luis Fallas. La visita funcionó como una observación directa de los alojamientos (ranchones), donde la delegación constató viviendas inundadas y casos activos de malaria.
-El evento se destaca por su impacto en la perspectiva legislativa del Ministro. Tras presenciar las condiciones y el confinamiento de los trabajadores, León Herrera admitió explícitamente una divergencia entre lo "legal" y lo "justo".</t>
-  </si>
-  <si>
-    <t>sabotage_1934</t>
-  </si>
-  <si>
-    <t>Countermanded Order of Sabotage</t>
-  </si>
-  <si>
-    <t>Contraorden de sabotaje</t>
-  </si>
-  <si>
-    <t>During a period of heightened tension in the 1934 strike, Carlos Luis Fallas—acting on unverified intelligence regarding approaching authorities—issued a written order to destroy a bridge to impede troop movement. Jaime Cerdas, co-leader of the movement, disputed the decision and unilaterally issued a countermand, nullifying the sabotage order without Fallas's immediate knowledge.</t>
-  </si>
-  <si>
-    <t>Durante un periodo de alta tensión en la huelga de 1934, Carlos Luis Fallas—actuando bajo inteligencia no verificada sobre el avance de las autoridades—emitió una orden escrita para destruir un puente y así impedir el movimiento de tropas. Jaime Cerdas, codirigente del movimiento, cuestionó la decisión y emitió unilateralmente una contraorden, anulando el sabotaje sin el conocimiento inmediato de Fallas.</t>
-  </si>
-  <si>
-    <t>Malaria Outbreak: Guápiles Sector</t>
-  </si>
-  <si>
-    <t>Brote de malaria: Sector Guápiles</t>
-  </si>
-  <si>
-    <t>migration</t>
-  </si>
-  <si>
-    <t>displacement</t>
-  </si>
-  <si>
-    <t>Sanitary Displacement: Guápiles to Siquirres</t>
-  </si>
-  <si>
-    <t>Desplazamiento sanitario: De Guápiles a Siquirres</t>
-  </si>
-  <si>
-    <t>Malaria Outbreak: Remote Plantations</t>
-  </si>
-  <si>
-    <t>Brote de malaria: Fincas remotas</t>
-  </si>
-  <si>
-    <t>Desplazamiento sanitario: Fincas remotas a Limón</t>
-  </si>
-  <si>
-    <t>Sanitary Displacement: Remote Plantations to Limón</t>
-  </si>
-  <si>
-    <t>Jaime Cerdas Mora reports a lack of medical infrastructure in the Guápiles sector. He notes that there were no resident doctors or local hospitals, leaving workers without immediate care during malaria outbreaks.</t>
-  </si>
-  <si>
-    <t>Jaime Cerdas Mora informa sobre la falta de infraestructura médica en el sector de Guápiles. Señala que no había médicos residentes ni hospitales locales, lo que dejaba a los trabajadores sin atención inmediata durante los brotes de malaria.</t>
-  </si>
-  <si>
-    <t>Jaime Cerdas Mora states that in remote plantations, malaria cases were frequent due to workers living in flooded barracks (ranchones). He estimates that half of the workers were unable to work half of the time because of the disease.</t>
-  </si>
-  <si>
-    <t>Jaime Cerdas Mora afirma que en fincas remotas, los casos de malaria eran frecuentes debido a que los trabajadores vivían en barracones (ranchones) inundados. Estima que la mitad de los trabajadores no podía laborar la mitad del tiempo a causa de la enfermedad.</t>
-  </si>
-  <si>
-    <t>Cerdas describes workers from Guápiles traveling to Siquirres for treatment. He identifies the facility there as a dispensary staffed by a nurse rather than a doctor, where quinine was the only medicine provided.</t>
-  </si>
-  <si>
-    <t>Cerdas describe a los trabajadores de Guápiles viajando a Siquirres para recibir tratamiento. Identifica la instalación allí como un dispensario atendido por un enfermero en lugar de un médico, donde la quinina era el único medicamento suministrado.</t>
-  </si>
-  <si>
-    <t>Cerdas explains that workers in remote areas, such as those near the Sixaola river, were forced to travel to the city of Limón to find a hospital. This required sick laborers to travel long distances from the plantations to the provincial capital.</t>
-  </si>
-  <si>
-    <t>Cerdas explica que los trabajadores de zonas remotas, como las cercanas al río Sixaola, se veían obligados a trasladarse a la ciudad de Limón para encontrar un hospital. Esto requería que los obreros enfermos viajaran largas distancias desde las fincas hasta la capital provincial.</t>
-  </si>
-  <si>
-    <t>Judicial Confinement of Carlos Luis Fallas to Limón</t>
-  </si>
-  <si>
-    <t>Confinamiento judicial de Carlos Luis Fallas a Limón</t>
-  </si>
-  <si>
-    <t>Based on the account by Jaime Cerdas Mora, the Communist Party drafted a formal list of demands (pliego de peticiones) and organized strike committees across the various banana plantations. The document was presented to the manager of the United Fruit Company, George P. Chittenden, who refused to receive it.</t>
-  </si>
-  <si>
-    <t>declaration_strike_1934</t>
-  </si>
-  <si>
-    <t>demands_strike_1934</t>
-  </si>
-  <si>
-    <t>Según el relato de Jaime Cerdas Mora, el Partido Comunista redactó un pliego de peticiones formal y organizó comités de huelga en las diversas fincas bananeras. El documento fue presentado al gerente de la United Fruit Company, George P. Chittenden, quien se negó a recibirlo.</t>
-  </si>
-  <si>
-    <t>Leadership Deployment to 26 Millas</t>
-  </si>
-  <si>
-    <t>Despliegue de la dirigencia hacia 26 Millas</t>
-  </si>
-  <si>
-    <t>movement</t>
-  </si>
-  <si>
-    <t>Following a strike organized in Alajuela, judicial authorities sentenced Carlos Luis Fallas to confinement (confinamiento) in Limón, where he arrives in December 1933. This was a common legal penalty at the time, used to isolate political and labor leaders from their active organizational bases. While in Limón, Fallas utilized his previous experience working for the banana companies to inform the Communist Party leadership in San José about the labor and sanitary conditions in the Atlantic zone.</t>
-  </si>
-  <si>
-    <t>Tras una huelga que organizó en Alajuela, las autoridades judiciales sentenciaron a Carlos Luis Fallas a la pena de confinamiento en Limón, adonde llega en diciembre de 1933. Esta era una sanción legal común en la época, utilizada para aislar a líderes políticos y sindicales de sus bases organizativas activas. Durante su estancia en Limón, Fallas aprovechó su experiencia previa trabajando para las bananeras para informar a la dirigencia del Partido Comunista en San José sobre las condiciones laborales y sanitarias en la zona atlántica.</t>
-  </si>
-  <si>
-    <t>Los comisariatos y la doble explotación obrera</t>
-  </si>
-  <si>
-    <t>comisariatos_1934_strike</t>
-  </si>
-  <si>
-    <t>Los comisariatos vinculados a la UFCo y a las fincas bananeras formaban un sistema de dependencia económica a lo largo de la zona bananera atlántica. Con frecuencia, los trabajadores eran pagados mediante cupones o chapas que solo podían utilizarse en los comisariatos de las plantaciones, donde los productos se vendían a precios elevados. Según el relato de Jaime Cerdas, este sistema agravaba los bajos salarios y las malas condiciones de vida, produciendo una “doble explotación” de los trabajadores bananeros a través tanto del trabajo como del consumo controlado.</t>
-  </si>
-  <si>
-    <t>UFCo and plantation-linked comisariatos formed a system of economic dependency across the Atlantic banana zone. Workers were frequently paid with coupons or tokens redeemable only at plantation commissaries, where goods were sold at inflated prices. According to Jaime Cerdas, this arrangement compounded already poor wages and living conditions, reinforcing what he described as a “double exploitation” of banana workers through both labor and controlled consumption.</t>
-  </si>
-  <si>
-    <t>Commissaries and the Double Exploitation of Workers</t>
-  </si>
-  <si>
-    <t>Declaration of Strike</t>
-  </si>
-  <si>
-    <t>1934_strike_marker_003</t>
-  </si>
-  <si>
-    <t>worker_meeting_01_1934</t>
-  </si>
-  <si>
-    <t>87–88</t>
-  </si>
-  <si>
-    <t>Paralysis of the Atlantic Region</t>
-  </si>
-  <si>
-    <t>La paralización de la zona atlántica</t>
-  </si>
-  <si>
-    <t>Declaración de la huelga</t>
-  </si>
-  <si>
-    <t>By the day following its formal declaration, the 1934 banana strike had spread across the Atlantic banana zone. According to Jaime Cerdas, plantations throughout the region had already joined the movement, paralyzing production, transportation, and UFCo operations across the corridor.</t>
-  </si>
-  <si>
-    <t>Para el día siguiente de su declaración formal, la huelga bananera de 1934 ya se había extendido por toda la zona bananera atlántica. Según Jaime Cerdas, plantaciones a lo largo de la región se habían incorporado al movimiento, paralizando la producción, el transporte y las operaciones de la UFCo en todo el corredor bananero.</t>
-  </si>
-  <si>
-    <t>Following the rejection of the workers’ petition by UFCo manager George P. Chittenden. Workers held a meeting around August 7, 1934 and agreed to go on strike. Strike committees had already been organized across multiple plantations, and Carlos Luis Fallas and Jaime Cerdas were tasked with directing the movement. Traveling by train to Madre de Dios and then on foot toward  26 Millas, they established the principal operational headquarters of the strike near the finca Los Ángeles. According to Cerdas’ account, delegations from plantations across the Atlantic banana corridor were already gathering there upon their arrival.</t>
-  </si>
-  <si>
-    <t>Tras el rechazo del pliego de peticiones de los trabajadores por parte del gerente de la UFCo, George P. Chittenden. Los obreros sostuvieron una reunión cerca del 7 de agosto de 1934, en la que se acordó ir a huelga. Para entonces, ya se habían organizado comités de huelga en múltiples plantaciones, y Carlos Luis Fallas y Jaime Cerdas fueron encargados de dirigir el movimiento. Viajando en tren hasta Madre de Dios y luego a pie hacia 26 Millas, establecieron el principal cuartel operativo de la huelga cerca de la finca Los Ángeles. Según el relato de Cerdas, delegaciones de plantaciones a lo largo del corredor bananero atlántico ya se estaban reuniendo allí al momento de su llegada.</t>
-  </si>
-  <si>
-    <t>On August 9, 1934, strike leaders formally declared the beginning of the banana strike. The declaration marked the transition from localized labor grievances to a coordinated regional movement across the Atlantic banana zone.</t>
-  </si>
-  <si>
-    <t>El 9 de agosto de 1934, los dirigentes huelguistas declararon formalmente el inicio de la huelga bananera. La declaración marcó la transición de reclamos laborales localizados hacia un movimiento coordinado a escala regional en la zona bananera atlántica.</t>
-  </si>
-  <si>
-    <t>Deposition of Carlos Luis Fallas</t>
-  </si>
-  <si>
-    <t>Deposición de Carlos Luis Fallas</t>
-  </si>
-  <si>
-    <t>Presentación y rechazo del pliego de peticiones</t>
-  </si>
-  <si>
-    <t>Presentation and Rejection of the List of Demands</t>
-  </si>
-  <si>
-    <t>Cuartel general de los huelguistas durante la huelga bananera de 1934.</t>
-  </si>
-  <si>
-    <t>action</t>
-  </si>
-  <si>
-    <t>exploitation</t>
-  </si>
-  <si>
-    <t>public_site</t>
+El evento se destaca por su impacto en la perspectiva del Ministro. Tras presenciar las condiciones y el confinamiento de los trabajadores, León Herrera admitió explícitamente una divergencia entre lo "legal" y lo "justo".</t>
+  </si>
+  <si>
+    <t>Huelga bananera de 1934</t>
+  </si>
+  <si>
+    <t>Following the rejection of the workers’ petition by UFCo manager George P. Chittenden. Workers held a meeting around August 7, 1934 and agreed to go on strike. Strike committees had already been organized across multiple plantations, and Carlos Luis Fallas and Jaime Cerdas were tasked with directing the movement. Traveling by train to Madre de Dios and then on foot toward  26 Millas, they established the principal operational headquarters of the strike near the Los Ángeles plantation. According to Cerdas’ account, delegations from plantations across the Atlantic banana corridor were already gathering there upon their arrival.</t>
+  </si>
+  <si>
+    <t>finca_la_fortuna</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>countermanded_sabotage_1934</t>
+  </si>
+  <si>
+    <t>Conflict Between Fallas and Lino Bustos</t>
+  </si>
+  <si>
+    <t>Conflicto entre Fallas y Lino Bustos</t>
+  </si>
+  <si>
+    <t>confrontation</t>
+  </si>
+  <si>
+    <t>lino_bustos</t>
+  </si>
+  <si>
+    <t>Lino Bustos</t>
+  </si>
+  <si>
+    <t>fallas-bustos_conflict_1934</t>
+  </si>
+  <si>
+    <t>During the 1934 banana strike, tensions emerged within the strike movement itself when Carlos Luis Fallas became involved in a heated confrontation with a worker named Lino Bustos, described by Jaime Cerdas as an admirer of Fallas. According to Cerdas, the argument escalated to the point that Bustos drew a knife and began threatening Fallas before the situation dissipated. The incident illustrates the internal pressures and personal conflicts that developed within the rapidly expanding strike movement.</t>
+  </si>
+  <si>
+    <t>Durante la huelga bananera de 1934, surgieron tensiones dentro del propio movimiento huelguístico cuando Carlos Luis Fallas se vio involucrado en una fuerte confrontación con un trabajador llamado Lino Bustos, descrito por Jaime Cerdas como admirador de Fallas. Según Cerdas, la discusión escaló hasta el punto en que Bustos sacó un cuchillo y comenzó a amenazar a Fallas antes de que la situación se disipara. El incidente refleja las presiones internas y los conflictos personales que surgieron dentro del movimiento huelguístico en rápida expansión.</t>
+  </si>
+  <si>
+    <t>worker</t>
+  </si>
+  <si>
+    <t>Fallas Travels to Dos Bocas</t>
+  </si>
+  <si>
+    <t>Fallas viaja a Dos Bocas</t>
+  </si>
+  <si>
+    <t>fallas_to_dos_bocas_1934</t>
+  </si>
+  <si>
+    <t>Following the confrontation with Lino Bustos, Carlos Luis Fallas departed for Dos Bocas while strike coordination efforts continued across the Atlantic banana zone. His movement formed part of the broader organizational activity through which strike leaders traveled between plantations and camps to maintain communication and direction during the conflict.</t>
+  </si>
+  <si>
+    <t>Tras la confrontación con Lino Bustos, Carlos Luis Fallas partió hacia Dos Bocas mientras continuaban los esfuerzos de coordinación de la huelga en la zona bananera atlántica. Su desplazamiento formó parte de la actividad organizativa más amplia mediante la cual los dirigentes huelguísticos se movilizaban entre plantaciones y campamentos para mantener la comunicación y la dirección del movimiento.</t>
+  </si>
+  <si>
+    <t>bustos_to_la_fortuna_1934</t>
+  </si>
+  <si>
+    <t>Lino Bustos Sent to La Fortuna</t>
+  </si>
+  <si>
+    <t>Lino Bustos enviado a La Fortuna</t>
+  </si>
+  <si>
+    <t>Amid fears that the company might orchestrate acts of sabotage to discredit the strike movement, Jaime Cerdas received reports of possible threats at the plantation of La Fortuna. Taking advantage of the situation following Bustos’ conflict with Fallas, Cerdas assigned Lino Bustos to travel to La Fortuna and oversee the protection of company property and plantation operations in the area.</t>
+  </si>
+  <si>
+    <t>En medio de temores de que la compañía pudiera organizar actos de sabotaje para desacreditar al movimiento huelguístico, Jaime Cerdas recibió informes sobre posibles amenazas en la finca La Fortuna. Aprovechando la situación tras el conflicto entre Bustos y Fallas, Cerdas asignó a Lino Bustos la tarea de trasladarse a La Fortuna para supervisar la protección de la propiedad de la compañía y de las operaciones de la plantación en la zona.</t>
+  </si>
+  <si>
+    <t>company_town</t>
+  </si>
+  <si>
+    <t>Based on the account by Jaime Cerdas Mora, the Communist Party drafted a formal list of demands and organized strike committees across the various banana plantations. The document was presented to the manager of the United Fruit Company, George P. Chittenden, who refused to receive it.</t>
+  </si>
+  <si>
+    <t>As the 1934 banana strike expanded across the Atlantic zone, local authorities attempted to suppress the movement by ordering the arrest of striking workers traveling along public roads. According to Jaime Cerdas, these measures sought to disrupt communication and mobility between plantations participating in the strike.</t>
+  </si>
+  <si>
+    <t>Durante la huelga, Manuel Mora utilizó su inmunidad legislativa para evitar ser arrestado mientras operaba en Siquirres, donde presentó recursos de habeas corpus para obtener la liberación de trabajadores detenidos. Según Jaime Cerdas, la posición legal y política de Mora le permitió continuar coordinando apoyo para el movimiento a pesar de la represión gubernamental.</t>
+  </si>
+  <si>
+    <t>In an effort to weaken the strike, authorities deployed police forces to cut and transport bananas in place of striking workers. The measure formed part of broader attempts by the government and the company to maintain banana production and contain the paralysis of the Atlantic banana zone.</t>
+  </si>
+  <si>
+    <t>En un intento por debilitar la huelga, las autoridades desplegaron fuerzas policiales para cortar y transportar banano en sustitución de los trabajadores huelguistas. La medida formó parte de esfuerzos más amplios del gobierno y la compañía por mantener la producción bananera y contener la paralización de la zona bananera atlántica.</t>
+  </si>
+  <si>
+    <t>In response to the use of police labor, striking workers organized nighttime actions to destroy banana production near the plantations. According to Jaime Cerdas, workers overturned approximately ten hectares of banana fields, ensuring that no quality bananas reached Limón for export.</t>
+  </si>
+  <si>
+    <t>En respuesta al uso de fuerzas policiales como mano de obra, trabajadores huelguistas organizaron acciones nocturnas para destruir producción bananera cerca de las plantaciones. Según Jaime Cerdas, los trabajadores derribaron aproximadamente diez hectáreas de banano, asegurando que ningún banano de calidad llegara a Limón para su exportación.</t>
+  </si>
+  <si>
+    <t>violence</t>
+  </si>
+  <si>
+    <t>santos_leon_herrera</t>
+  </si>
+  <si>
+    <t>Santos León Herrera</t>
+  </si>
+  <si>
+    <t>official</t>
+  </si>
+  <si>
+    <t>Minister of Government and Labor (1932–1936)</t>
+  </si>
+  <si>
+    <t>Ministro de Gobernación y Trabajo (1932–1936)</t>
   </si>
 </sst>
 </file>
@@ -1130,8 +1211,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8DE4AF77-3078-41E5-A862-A672CD070CDC}" name="Table2" displayName="Table2" ref="A1:Y66" totalsRowShown="0">
-  <autoFilter ref="A1:Y66" xr:uid="{8DE4AF77-3078-41E5-A862-A672CD070CDC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8DE4AF77-3078-41E5-A862-A672CD070CDC}" name="Table2" displayName="Table2" ref="A1:Y71" totalsRowShown="0">
+  <autoFilter ref="A1:Y71" xr:uid="{8DE4AF77-3078-41E5-A862-A672CD070CDC}"/>
   <tableColumns count="25">
     <tableColumn id="1" xr3:uid="{BA8A667B-2EA1-408D-ABAE-261F71369134}" name="id"/>
     <tableColumn id="2" xr3:uid="{1E8557DA-5346-4170-9098-68F69CB64A7F}" name="label_en"/>
@@ -1480,10 +1561,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21EAC64A-5CB7-4B0B-817E-D41EE9B9A394}">
-  <dimension ref="A1:Y66"/>
+  <dimension ref="A1:Y71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="75.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="53.140625" customWidth="1"/>
     <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -1525,10 +1606,10 @@
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="G1" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="H1" t="s">
         <v>6</v>
@@ -1546,7 +1627,7 @@
         <v>5</v>
       </c>
       <c r="M1" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="N1" t="s">
         <v>8</v>
@@ -1567,16 +1648,16 @@
         <v>13</v>
       </c>
       <c r="T1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="U1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="V1" t="s">
         <v>15</v>
       </c>
       <c r="W1" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="X1" t="s">
         <v>14</v>
@@ -1611,7 +1692,7 @@
         <v>9.9281000000000006</v>
       </c>
       <c r="M2" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
@@ -1640,7 +1721,7 @@
         <v>10.0162</v>
       </c>
       <c r="M3" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
@@ -1669,7 +1750,7 @@
         <v>9.9002999999999997</v>
       </c>
       <c r="M4" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
@@ -1698,7 +1779,7 @@
         <v>9.9922000000000004</v>
       </c>
       <c r="M5" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
@@ -1727,7 +1808,7 @@
         <v>9.9901999999999997</v>
       </c>
       <c r="M6" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
@@ -1756,7 +1837,7 @@
         <v>42.360100000000003</v>
       </c>
       <c r="M7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
@@ -1785,7 +1866,7 @@
         <v>42.360300000000002</v>
       </c>
       <c r="M8" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
@@ -1814,7 +1895,7 @@
         <v>10.097</v>
       </c>
       <c r="M9" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
@@ -1843,7 +1924,7 @@
         <v>29.9499</v>
       </c>
       <c r="M10" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
@@ -1875,13 +1956,13 @@
         <v>10.050000000000001</v>
       </c>
       <c r="M11" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T11" t="s">
         <v>47</v>
       </c>
       <c r="U11" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="V11" t="b">
         <v>1</v>
@@ -1916,13 +1997,13 @@
         <v>10.02</v>
       </c>
       <c r="M12" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T12" t="s">
         <v>45</v>
       </c>
       <c r="U12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
@@ -1954,13 +2035,13 @@
         <v>10.08</v>
       </c>
       <c r="M13" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T13" t="s">
         <v>45</v>
       </c>
       <c r="U13" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
@@ -1992,13 +2073,13 @@
         <v>10.1</v>
       </c>
       <c r="M14" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T14" t="s">
         <v>45</v>
       </c>
       <c r="U14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
@@ -2030,13 +2111,13 @@
         <v>9.9</v>
       </c>
       <c r="M15" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T15" t="s">
         <v>46</v>
       </c>
       <c r="U15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
@@ -2053,7 +2134,7 @@
         <v>24</v>
       </c>
       <c r="E16" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="H16">
         <v>1934</v>
@@ -2071,13 +2152,13 @@
         <v>10.0877643</v>
       </c>
       <c r="M16" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T16" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="U16" t="s">
-        <v>289</v>
+        <v>269</v>
       </c>
       <c r="X16" t="s">
         <v>114</v>
@@ -2106,13 +2187,13 @@
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T17" t="s">
         <v>71</v>
       </c>
       <c r="U17" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="X17" t="s">
         <v>114</v>
@@ -2144,7 +2225,13 @@
         <v>10.094110000000001</v>
       </c>
       <c r="M18" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="X18" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y18">
+        <v>87</v>
       </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
@@ -2173,7 +2260,7 @@
         <v>10.215439999999999</v>
       </c>
       <c r="M19" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
@@ -2189,6 +2276,9 @@
       <c r="D20" t="s">
         <v>24</v>
       </c>
+      <c r="E20" t="s">
+        <v>306</v>
+      </c>
       <c r="J20" t="b">
         <v>1</v>
       </c>
@@ -2199,15 +2289,15 @@
         <v>10.28565</v>
       </c>
       <c r="M20" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>129</v>
+        <v>284</v>
       </c>
       <c r="B21" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C21" t="s">
         <v>60</v>
@@ -2222,21 +2312,30 @@
         <v>1</v>
       </c>
       <c r="K21">
-        <v>-83.790189999999996</v>
+        <v>-82.994263000000004</v>
       </c>
       <c r="L21">
-        <v>10.510669999999999</v>
+        <v>9.7301959999999994</v>
       </c>
       <c r="M21" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="N21" t="s">
+        <v>285</v>
+      </c>
+      <c r="X21" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y21">
+        <v>90</v>
       </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B22" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C22" t="s">
         <v>61</v>
@@ -2257,15 +2356,15 @@
         <v>10.17947</v>
       </c>
       <c r="M22" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>132</v>
+      </c>
+      <c r="B23" t="s">
         <v>133</v>
-      </c>
-      <c r="B23" t="s">
-        <v>134</v>
       </c>
       <c r="C23" t="s">
         <v>62</v>
@@ -2286,7 +2385,7 @@
         <v>10.086040000000001</v>
       </c>
       <c r="M23" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.25">
@@ -2315,7 +2414,7 @@
         <v>10.08187</v>
       </c>
       <c r="M24" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
@@ -2323,7 +2422,7 @@
         <v>65</v>
       </c>
       <c r="B25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C25" t="s">
         <v>66</v>
@@ -2344,13 +2443,13 @@
         <v>9.5016700000000007</v>
       </c>
       <c r="M25" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T25" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="U25" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="X25" t="s">
         <v>114</v>
@@ -2361,13 +2460,13 @@
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>135</v>
+      </c>
+      <c r="B26" t="s">
         <v>136</v>
       </c>
-      <c r="B26" t="s">
-        <v>137</v>
-      </c>
       <c r="C26" t="s">
-        <v>138</v>
+        <v>282</v>
       </c>
       <c r="D26" t="s">
         <v>72</v>
@@ -2394,7 +2493,7 @@
         <v>10.0877643</v>
       </c>
       <c r="M26" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="V26" t="b">
         <v>1</v>
@@ -2437,7 +2536,7 @@
         <v>83</v>
       </c>
       <c r="C28" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D28" t="s">
         <v>74</v>
@@ -2483,19 +2582,19 @@
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B30" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C30" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D30" t="s">
         <v>25</v>
       </c>
       <c r="E30" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H30">
         <v>1885</v>
@@ -2513,7 +2612,7 @@
         <v>-71.049722000000003</v>
       </c>
       <c r="M30" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
@@ -2536,7 +2635,7 @@
         <v>0</v>
       </c>
       <c r="M31" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
@@ -2544,10 +2643,10 @@
         <v>86</v>
       </c>
       <c r="B32" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C32" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D32" t="s">
         <v>74</v>
@@ -2559,7 +2658,7 @@
         <v>0</v>
       </c>
       <c r="M32" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.25">
@@ -2567,7 +2666,7 @@
         <v>107</v>
       </c>
       <c r="B33" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C33" t="s">
         <v>109</v>
@@ -2582,7 +2681,7 @@
         <v>0</v>
       </c>
       <c r="M33" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.25">
@@ -2590,7 +2689,7 @@
         <v>110</v>
       </c>
       <c r="B34" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C34" t="s">
         <v>111</v>
@@ -2605,7 +2704,7 @@
         <v>0</v>
       </c>
       <c r="M34" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.25">
@@ -2616,13 +2715,13 @@
         <v>87</v>
       </c>
       <c r="C35" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D35" t="s">
         <v>74</v>
       </c>
       <c r="E35" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="H35">
         <v>1931</v>
@@ -2631,7 +2730,7 @@
         <v>0</v>
       </c>
       <c r="M35" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.25">
@@ -2645,19 +2744,19 @@
         <v>91</v>
       </c>
       <c r="D36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E36" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="J36" t="b">
         <v>0</v>
       </c>
       <c r="T36" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="U36" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="V36" t="b">
         <v>1</v>
@@ -2674,10 +2773,10 @@
         <v>89</v>
       </c>
       <c r="D37" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E37" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="J37" t="b">
         <v>0</v>
@@ -2697,16 +2796,16 @@
         <v>94</v>
       </c>
       <c r="D38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E38" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="J38" t="b">
         <v>0</v>
       </c>
       <c r="M38" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="39" spans="1:25" x14ac:dyDescent="0.25">
@@ -2720,16 +2819,16 @@
         <v>105</v>
       </c>
       <c r="D39" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E39" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J39" t="b">
         <v>0</v>
       </c>
       <c r="M39" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.25">
@@ -2743,22 +2842,22 @@
         <v>96</v>
       </c>
       <c r="D40" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E40" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J40" t="b">
         <v>0</v>
       </c>
       <c r="M40" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T40" t="s">
         <v>103</v>
       </c>
       <c r="U40" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="X40" t="s">
         <v>114</v>
@@ -2778,22 +2877,22 @@
         <v>98</v>
       </c>
       <c r="D41" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E41" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="J41" t="b">
         <v>0</v>
       </c>
       <c r="M41" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T41" t="s">
         <v>103</v>
       </c>
       <c r="U41" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="X41" t="s">
         <v>114</v>
@@ -2813,22 +2912,22 @@
         <v>100</v>
       </c>
       <c r="D42" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E42" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="J42" t="b">
         <v>0</v>
       </c>
       <c r="M42" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T42" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="U42" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="X42" t="s">
         <v>114</v>
@@ -2848,172 +2947,109 @@
         <v>102</v>
       </c>
       <c r="D43" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E43" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="J43" t="b">
         <v>0</v>
       </c>
       <c r="M43" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="44" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>114</v>
+        <v>315</v>
       </c>
       <c r="B44" t="s">
-        <v>113</v>
+        <v>316</v>
       </c>
       <c r="C44" t="s">
-        <v>113</v>
+        <v>316</v>
       </c>
       <c r="D44" t="s">
-        <v>14</v>
+        <v>166</v>
       </c>
       <c r="E44" t="s">
-        <v>176</v>
-      </c>
-      <c r="H44">
-        <v>1984</v>
-      </c>
-      <c r="I44">
-        <v>1984</v>
+        <v>317</v>
       </c>
       <c r="J44" t="b">
-        <v>1</v>
-      </c>
-      <c r="K44" s="1">
-        <v>-84.090699999999998</v>
-      </c>
-      <c r="L44" s="1">
-        <v>9.9281000000000006</v>
+        <v>0</v>
       </c>
       <c r="M44" t="s">
-        <v>165</v>
-      </c>
-      <c r="V44" t="b">
-        <v>1</v>
-      </c>
-      <c r="W44" t="s">
-        <v>113</v>
-      </c>
-      <c r="X44" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y44">
-        <v>87</v>
+        <v>162</v>
+      </c>
+      <c r="T44" t="s">
+        <v>318</v>
+      </c>
+      <c r="U44" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="45" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>116</v>
+        <v>290</v>
       </c>
       <c r="B45" t="s">
-        <v>256</v>
+        <v>291</v>
       </c>
       <c r="C45" t="s">
-        <v>257</v>
+        <v>291</v>
       </c>
       <c r="D45" t="s">
-        <v>290</v>
+        <v>166</v>
       </c>
       <c r="E45" t="s">
-        <v>106</v>
-      </c>
-      <c r="F45" t="s">
-        <v>136</v>
-      </c>
-      <c r="G45">
-        <v>0</v>
-      </c>
-      <c r="H45">
-        <v>1933</v>
-      </c>
-      <c r="I45">
-        <v>1933</v>
+        <v>295</v>
       </c>
       <c r="J45" t="b">
         <v>0</v>
       </c>
       <c r="M45" t="s">
-        <v>165</v>
-      </c>
-      <c r="N45" t="s">
-        <v>67</v>
-      </c>
-      <c r="O45" t="s">
-        <v>18</v>
-      </c>
-      <c r="P45" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q45" t="s">
-        <v>110</v>
-      </c>
-      <c r="R45" t="s">
-        <v>104</v>
-      </c>
-      <c r="T45" t="s">
-        <v>265</v>
-      </c>
-      <c r="U45" t="s">
-        <v>266</v>
-      </c>
-      <c r="X45" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y45">
-        <v>86</v>
+        <v>162</v>
       </c>
     </row>
     <row r="46" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>170</v>
+        <v>114</v>
       </c>
       <c r="B46" t="s">
-        <v>244</v>
+        <v>113</v>
       </c>
       <c r="C46" t="s">
-        <v>245</v>
+        <v>113</v>
       </c>
       <c r="D46" t="s">
-        <v>72</v>
+        <v>14</v>
       </c>
       <c r="E46" t="s">
-        <v>175</v>
-      </c>
-      <c r="F46" t="s">
-        <v>136</v>
-      </c>
-      <c r="G46">
-        <v>1</v>
+        <v>173</v>
       </c>
       <c r="H46">
-        <v>1934</v>
+        <v>1984</v>
       </c>
       <c r="I46">
-        <v>1934</v>
+        <v>1984</v>
       </c>
       <c r="J46" t="b">
         <v>1</v>
       </c>
       <c r="K46" s="1">
-        <v>-82.9</v>
+        <v>-84.090699999999998</v>
       </c>
       <c r="L46" s="1">
-        <v>9.5500000000000007</v>
+        <v>9.9281000000000006</v>
       </c>
       <c r="M46" t="s">
-        <v>165</v>
-      </c>
-      <c r="T46" t="s">
-        <v>250</v>
-      </c>
-      <c r="U46" t="s">
-        <v>251</v>
+        <v>162</v>
+      </c>
+      <c r="V46" t="b">
+        <v>1</v>
+      </c>
+      <c r="W46" t="s">
+        <v>113</v>
       </c>
       <c r="X46" t="s">
         <v>114</v>
@@ -3024,78 +3060,90 @@
     </row>
     <row r="47" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>171</v>
+        <v>116</v>
       </c>
       <c r="B47" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="C47" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="D47" t="s">
-        <v>72</v>
+        <v>227</v>
       </c>
       <c r="E47" t="s">
-        <v>175</v>
+        <v>273</v>
       </c>
       <c r="F47" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H47">
-        <v>1934</v>
+        <v>1933</v>
       </c>
       <c r="I47">
-        <v>1934</v>
+        <v>1933</v>
       </c>
       <c r="J47" t="b">
-        <v>1</v>
-      </c>
-      <c r="K47" s="1">
-        <v>-83.791899999999998</v>
-      </c>
-      <c r="L47" s="1">
-        <v>10.217700000000001</v>
+        <v>0</v>
       </c>
       <c r="M47" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="N47" t="s">
+        <v>67</v>
+      </c>
+      <c r="O47" t="s">
+        <v>18</v>
+      </c>
+      <c r="P47" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>110</v>
+      </c>
+      <c r="R47" t="s">
+        <v>104</v>
+      </c>
+      <c r="S47" t="b">
+        <v>1</v>
       </c>
       <c r="T47" t="s">
-        <v>248</v>
+        <v>277</v>
       </c>
       <c r="U47" t="s">
-        <v>249</v>
+        <v>278</v>
       </c>
       <c r="X47" t="s">
         <v>114</v>
       </c>
       <c r="Y47">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="48" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B48" t="s">
-        <v>247</v>
+        <v>231</v>
       </c>
       <c r="C48" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="D48" t="s">
-        <v>240</v>
+        <v>72</v>
       </c>
       <c r="E48" t="s">
-        <v>241</v>
+        <v>172</v>
       </c>
       <c r="F48" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G48">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H48">
         <v>1934</v>
@@ -3104,25 +3152,22 @@
         <v>1934</v>
       </c>
       <c r="J48" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K48" s="1">
+        <v>-82.9</v>
+      </c>
+      <c r="L48" s="1">
+        <v>9.5500000000000007</v>
       </c>
       <c r="M48" t="s">
-        <v>165</v>
-      </c>
-      <c r="N48" t="s">
-        <v>170</v>
-      </c>
-      <c r="O48" t="s">
-        <v>18</v>
-      </c>
-      <c r="P48" t="b">
-        <v>1</v>
+        <v>162</v>
       </c>
       <c r="T48" t="s">
-        <v>254</v>
+        <v>237</v>
       </c>
       <c r="U48" t="s">
-        <v>255</v>
+        <v>238</v>
       </c>
       <c r="X48" t="s">
         <v>114</v>
@@ -3133,25 +3178,25 @@
     </row>
     <row r="49" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>168</v>
+      </c>
+      <c r="B49" t="s">
+        <v>225</v>
+      </c>
+      <c r="C49" t="s">
+        <v>226</v>
+      </c>
+      <c r="D49" t="s">
+        <v>72</v>
+      </c>
+      <c r="E49" t="s">
         <v>172</v>
       </c>
-      <c r="B49" t="s">
-        <v>242</v>
-      </c>
-      <c r="C49" t="s">
-        <v>243</v>
-      </c>
-      <c r="D49" t="s">
-        <v>240</v>
-      </c>
-      <c r="E49" t="s">
-        <v>241</v>
-      </c>
       <c r="F49" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H49">
         <v>1934</v>
@@ -3160,25 +3205,22 @@
         <v>1934</v>
       </c>
       <c r="J49" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K49" s="1">
+        <v>-83.791899999999998</v>
+      </c>
+      <c r="L49" s="1">
+        <v>10.217700000000001</v>
       </c>
       <c r="M49" t="s">
-        <v>165</v>
-      </c>
-      <c r="N49" t="s">
-        <v>171</v>
-      </c>
-      <c r="O49" t="s">
-        <v>27</v>
-      </c>
-      <c r="P49" t="b">
-        <v>1</v>
+        <v>162</v>
       </c>
       <c r="T49" t="s">
-        <v>252</v>
+        <v>235</v>
       </c>
       <c r="U49" t="s">
-        <v>253</v>
+        <v>236</v>
       </c>
       <c r="X49" t="s">
         <v>114</v>
@@ -3189,25 +3231,25 @@
     </row>
     <row r="50" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>268</v>
+        <v>170</v>
       </c>
       <c r="B50" t="s">
-        <v>271</v>
+        <v>234</v>
       </c>
       <c r="C50" t="s">
-        <v>267</v>
+        <v>233</v>
       </c>
       <c r="D50" t="s">
-        <v>72</v>
+        <v>227</v>
       </c>
       <c r="E50" t="s">
-        <v>291</v>
+        <v>228</v>
       </c>
       <c r="F50" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G50">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H50">
         <v>1934</v>
@@ -3216,48 +3258,54 @@
         <v>1934</v>
       </c>
       <c r="J50" t="b">
-        <v>1</v>
-      </c>
-      <c r="K50" s="1">
-        <v>-83.033799999999999</v>
-      </c>
-      <c r="L50" s="1">
-        <v>9.9901999999999997</v>
+        <v>0</v>
       </c>
       <c r="M50" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="N50" t="s">
+        <v>167</v>
+      </c>
+      <c r="O50" t="s">
+        <v>18</v>
+      </c>
+      <c r="P50" t="b">
+        <v>1</v>
       </c>
       <c r="T50" t="s">
-        <v>270</v>
+        <v>241</v>
       </c>
       <c r="U50" t="s">
-        <v>269</v>
+        <v>242</v>
       </c>
       <c r="X50" t="s">
         <v>114</v>
       </c>
+      <c r="Y50">
+        <v>87</v>
+      </c>
     </row>
     <row r="51" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>260</v>
+        <v>169</v>
       </c>
       <c r="B51" t="s">
-        <v>288</v>
+        <v>229</v>
       </c>
       <c r="C51" t="s">
-        <v>287</v>
+        <v>230</v>
       </c>
       <c r="D51" t="s">
-        <v>168</v>
+        <v>227</v>
       </c>
       <c r="E51" t="s">
-        <v>184</v>
+        <v>228</v>
       </c>
       <c r="F51" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G51">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H51">
         <v>1934</v>
@@ -3269,31 +3317,22 @@
         <v>0</v>
       </c>
       <c r="M51" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="N51" t="s">
-        <v>16</v>
+        <v>168</v>
       </c>
       <c r="O51" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="P51" t="b">
         <v>1</v>
       </c>
-      <c r="Q51" t="s">
-        <v>84</v>
-      </c>
-      <c r="R51" t="s">
-        <v>90</v>
-      </c>
-      <c r="S51" t="b">
-        <v>1</v>
-      </c>
       <c r="T51" t="s">
-        <v>258</v>
+        <v>239</v>
       </c>
       <c r="U51" t="s">
-        <v>261</v>
+        <v>240</v>
       </c>
       <c r="X51" t="s">
         <v>114</v>
@@ -3304,25 +3343,25 @@
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>251</v>
+      </c>
+      <c r="B52" t="s">
         <v>274</v>
       </c>
-      <c r="B52" t="s">
-        <v>262</v>
-      </c>
       <c r="C52" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="D52" t="s">
         <v>72</v>
       </c>
       <c r="E52" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="F52" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G52">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H52">
         <v>1934</v>
@@ -3331,25 +3370,22 @@
         <v>1934</v>
       </c>
       <c r="J52" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K52" s="1">
+        <v>-83.506900000000002</v>
+      </c>
+      <c r="L52" s="1">
+        <v>10.097</v>
       </c>
       <c r="M52" t="s">
-        <v>165</v>
-      </c>
-      <c r="N52" t="s">
-        <v>18</v>
-      </c>
-      <c r="O52" t="s">
-        <v>48</v>
-      </c>
-      <c r="P52" t="b">
-        <v>1</v>
+        <v>162</v>
       </c>
       <c r="T52" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="U52" t="s">
-        <v>282</v>
+        <v>252</v>
       </c>
       <c r="X52" t="s">
         <v>114</v>
@@ -3360,25 +3396,25 @@
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
       <c r="B53" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="C53" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="D53" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E53" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="F53" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G53">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H53">
         <v>1934</v>
@@ -3387,51 +3423,63 @@
         <v>1934</v>
       </c>
       <c r="J53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M53" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="N53" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="O53" t="s">
         <v>17</v>
       </c>
+      <c r="P53" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q53" t="s">
+        <v>84</v>
+      </c>
+      <c r="R53" t="s">
+        <v>90</v>
+      </c>
+      <c r="S53" t="b">
+        <v>1</v>
+      </c>
       <c r="T53" t="s">
-        <v>283</v>
+        <v>307</v>
       </c>
       <c r="U53" t="s">
-        <v>284</v>
+        <v>247</v>
       </c>
       <c r="X53" t="s">
         <v>114</v>
       </c>
-      <c r="Y53" t="s">
-        <v>275</v>
+      <c r="Y53">
+        <v>87</v>
       </c>
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>273</v>
+        <v>255</v>
       </c>
       <c r="B54" t="s">
-        <v>276</v>
+        <v>248</v>
       </c>
       <c r="C54" t="s">
-        <v>277</v>
+        <v>249</v>
       </c>
       <c r="D54" t="s">
         <v>72</v>
       </c>
       <c r="E54" t="s">
-        <v>73</v>
+        <v>250</v>
       </c>
       <c r="F54" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G54">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H54">
         <v>1934</v>
@@ -3440,51 +3488,54 @@
         <v>1934</v>
       </c>
       <c r="J54" t="b">
-        <v>1</v>
-      </c>
-      <c r="K54">
-        <v>-83.355490700000004</v>
-      </c>
-      <c r="L54">
-        <v>10.0877643</v>
+        <v>0</v>
       </c>
       <c r="M54" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="N54" t="s">
+        <v>18</v>
+      </c>
+      <c r="O54" t="s">
+        <v>48</v>
+      </c>
+      <c r="P54" t="b">
+        <v>1</v>
       </c>
       <c r="T54" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="U54" t="s">
-        <v>280</v>
+        <v>262</v>
       </c>
       <c r="X54" t="s">
         <v>114</v>
       </c>
       <c r="Y54">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="55" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>118</v>
+        <v>245</v>
       </c>
       <c r="B55" t="s">
-        <v>223</v>
+        <v>253</v>
       </c>
       <c r="C55" t="s">
-        <v>146</v>
+        <v>259</v>
       </c>
       <c r="D55" t="s">
-        <v>290</v>
+        <v>165</v>
       </c>
       <c r="E55" t="s">
-        <v>106</v>
+        <v>181</v>
       </c>
       <c r="F55" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G55">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H55">
         <v>1934</v>
@@ -3493,60 +3544,51 @@
         <v>1934</v>
       </c>
       <c r="J55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M55" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="N55" t="s">
-        <v>119</v>
+        <v>48</v>
       </c>
       <c r="O55" t="s">
-        <v>27</v>
-      </c>
-      <c r="P55" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q55" t="s">
-        <v>93</v>
-      </c>
-      <c r="R55" t="s">
-        <v>117</v>
+        <v>17</v>
       </c>
       <c r="T55" t="s">
-        <v>162</v>
+        <v>263</v>
       </c>
       <c r="U55" t="s">
-        <v>161</v>
+        <v>264</v>
       </c>
       <c r="X55" t="s">
         <v>114</v>
       </c>
-      <c r="Y55">
-        <v>88</v>
+      <c r="Y55" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="56" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>119</v>
+        <v>254</v>
       </c>
       <c r="B56" t="s">
-        <v>222</v>
+        <v>257</v>
       </c>
       <c r="C56" t="s">
-        <v>145</v>
+        <v>258</v>
       </c>
       <c r="D56" t="s">
-        <v>290</v>
+        <v>72</v>
       </c>
       <c r="E56" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
       <c r="F56" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G56">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H56">
         <v>1934</v>
@@ -3557,29 +3599,20 @@
       <c r="J56" t="b">
         <v>1</v>
       </c>
-      <c r="K56" s="1">
-        <v>-83.54</v>
-      </c>
-      <c r="L56" s="1">
-        <v>10.1</v>
+      <c r="K56">
+        <v>-83.355490700000004</v>
+      </c>
+      <c r="L56">
+        <v>10.0877643</v>
       </c>
       <c r="M56" t="s">
-        <v>165</v>
-      </c>
-      <c r="P56" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q56" t="s">
-        <v>107</v>
-      </c>
-      <c r="R56" t="s">
-        <v>136</v>
+        <v>162</v>
       </c>
       <c r="T56" t="s">
-        <v>211</v>
+        <v>260</v>
       </c>
       <c r="U56" t="s">
-        <v>163</v>
+        <v>261</v>
       </c>
       <c r="X56" t="s">
         <v>114</v>
@@ -3590,25 +3623,25 @@
     </row>
     <row r="57" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>186</v>
+        <v>118</v>
       </c>
       <c r="B57" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="C57" t="s">
-        <v>188</v>
+        <v>144</v>
       </c>
       <c r="D57" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
       <c r="E57" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F57" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G57">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H57">
         <v>1934</v>
@@ -3620,28 +3653,31 @@
         <v>0</v>
       </c>
       <c r="M57" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="N57" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="O57" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="P57" t="b">
         <v>1</v>
       </c>
       <c r="Q57" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="R57" t="s">
-        <v>136</v>
+        <v>117</v>
+      </c>
+      <c r="S57" t="b">
+        <v>1</v>
       </c>
       <c r="T57" t="s">
-        <v>190</v>
+        <v>160</v>
       </c>
       <c r="U57" t="s">
-        <v>189</v>
+        <v>159</v>
       </c>
       <c r="X57" t="s">
         <v>114</v>
@@ -3652,25 +3688,25 @@
     </row>
     <row r="58" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>187</v>
+        <v>119</v>
       </c>
       <c r="B58" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="C58" t="s">
-        <v>192</v>
+        <v>143</v>
       </c>
       <c r="D58" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
       <c r="E58" t="s">
-        <v>191</v>
+        <v>108</v>
       </c>
       <c r="F58" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G58">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="H58">
         <v>1934</v>
@@ -3682,28 +3718,31 @@
         <v>0</v>
       </c>
       <c r="M58" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="N58" t="s">
+        <v>27</v>
+      </c>
+      <c r="O58" t="s">
         <v>48</v>
       </c>
-      <c r="O58" t="s">
-        <v>18</v>
-      </c>
       <c r="P58" t="b">
         <v>1</v>
       </c>
       <c r="Q58" t="s">
-        <v>136</v>
+        <v>107</v>
       </c>
       <c r="R58" t="s">
-        <v>107</v>
+        <v>135</v>
+      </c>
+      <c r="S58" t="b">
+        <v>1</v>
       </c>
       <c r="T58" t="s">
-        <v>209</v>
+        <v>308</v>
       </c>
       <c r="U58" t="s">
-        <v>208</v>
+        <v>309</v>
       </c>
       <c r="X58" t="s">
         <v>114</v>
@@ -3714,25 +3753,25 @@
     </row>
     <row r="59" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>219</v>
+        <v>183</v>
       </c>
       <c r="B59" t="s">
-        <v>285</v>
+        <v>211</v>
       </c>
       <c r="C59" t="s">
-        <v>286</v>
+        <v>185</v>
       </c>
       <c r="D59" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
       <c r="E59" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F59" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G59">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H59">
         <v>1934</v>
@@ -3744,92 +3783,125 @@
         <v>0</v>
       </c>
       <c r="M59" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="N59" t="s">
+        <v>27</v>
+      </c>
+      <c r="O59" t="s">
         <v>48</v>
       </c>
-      <c r="O59" t="s">
-        <v>210</v>
-      </c>
       <c r="P59" t="b">
         <v>1</v>
       </c>
+      <c r="Q59" t="s">
+        <v>107</v>
+      </c>
+      <c r="R59" t="s">
+        <v>135</v>
+      </c>
+      <c r="S59" t="b">
+        <v>1</v>
+      </c>
       <c r="T59" t="s">
-        <v>218</v>
+        <v>310</v>
       </c>
       <c r="U59" t="s">
-        <v>217</v>
+        <v>311</v>
       </c>
       <c r="X59" t="s">
         <v>114</v>
       </c>
       <c r="Y59">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="60" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>184</v>
+      </c>
+      <c r="B60" t="s">
         <v>210</v>
       </c>
-      <c r="B60" t="s">
-        <v>213</v>
-      </c>
       <c r="C60" t="s">
-        <v>213</v>
+        <v>186</v>
       </c>
       <c r="D60" t="s">
-        <v>24</v>
+        <v>270</v>
       </c>
       <c r="E60" t="s">
-        <v>292</v>
+        <v>314</v>
+      </c>
+      <c r="F60" t="s">
+        <v>135</v>
+      </c>
+      <c r="G60">
+        <v>11</v>
       </c>
       <c r="H60">
-        <v>1855</v>
+        <v>1934</v>
       </c>
       <c r="I60">
-        <v>1958</v>
+        <v>1934</v>
       </c>
       <c r="J60" t="b">
-        <v>1</v>
-      </c>
-      <c r="K60">
-        <v>-84.085564000000005</v>
-      </c>
-      <c r="L60">
-        <v>9.9354469999999999</v>
+        <v>0</v>
       </c>
       <c r="M60" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="N60" t="s">
+        <v>48</v>
+      </c>
+      <c r="O60" t="s">
+        <v>27</v>
+      </c>
+      <c r="P60" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>135</v>
+      </c>
+      <c r="R60" t="s">
+        <v>107</v>
+      </c>
+      <c r="S60" t="b">
+        <v>1</v>
       </c>
       <c r="T60" t="s">
-        <v>214</v>
+        <v>312</v>
       </c>
       <c r="U60" t="s">
-        <v>225</v>
+        <v>313</v>
+      </c>
+      <c r="X60" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y60">
+        <v>88</v>
       </c>
     </row>
     <row r="61" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B61" t="s">
-        <v>226</v>
+        <v>265</v>
       </c>
       <c r="C61" t="s">
-        <v>227</v>
+        <v>266</v>
       </c>
       <c r="D61" t="s">
-        <v>72</v>
+        <v>270</v>
       </c>
       <c r="E61" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
       <c r="F61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G61">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H61">
         <v>1934</v>
@@ -3838,22 +3910,25 @@
         <v>1934</v>
       </c>
       <c r="J61" t="b">
-        <v>1</v>
-      </c>
-      <c r="K61">
-        <v>-84.085564000000005</v>
-      </c>
-      <c r="L61">
-        <v>9.9354469999999999</v>
+        <v>0</v>
       </c>
       <c r="M61" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="N61" t="s">
+        <v>48</v>
+      </c>
+      <c r="O61" t="s">
+        <v>202</v>
+      </c>
+      <c r="P61" t="b">
+        <v>1</v>
       </c>
       <c r="T61" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="U61" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="X61" t="s">
         <v>114</v>
@@ -3864,81 +3939,66 @@
     </row>
     <row r="62" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>228</v>
+        <v>202</v>
       </c>
       <c r="B62" t="s">
-        <v>229</v>
+        <v>204</v>
       </c>
       <c r="C62" t="s">
-        <v>230</v>
+        <v>204</v>
       </c>
       <c r="D62" t="s">
-        <v>290</v>
+        <v>24</v>
       </c>
       <c r="E62" t="s">
-        <v>106</v>
-      </c>
-      <c r="F62" t="s">
-        <v>136</v>
-      </c>
-      <c r="G62">
-        <v>13</v>
+        <v>272</v>
       </c>
       <c r="H62">
-        <v>1934</v>
+        <v>1855</v>
       </c>
       <c r="I62">
-        <v>1934</v>
+        <v>1958</v>
       </c>
       <c r="J62" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K62">
+        <v>-84.085564000000005</v>
+      </c>
+      <c r="L62">
+        <v>9.9354469999999999</v>
       </c>
       <c r="M62" t="s">
-        <v>165</v>
-      </c>
-      <c r="N62" t="s">
-        <v>210</v>
-      </c>
-      <c r="O62" t="s">
-        <v>48</v>
-      </c>
-      <c r="P62" t="b">
-        <v>1</v>
+        <v>162</v>
       </c>
       <c r="T62" t="s">
-        <v>231</v>
+        <v>205</v>
       </c>
       <c r="U62" t="s">
-        <v>232</v>
-      </c>
-      <c r="X62" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y62">
-        <v>89</v>
+        <v>215</v>
       </c>
     </row>
     <row r="63" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>233</v>
+        <v>203</v>
       </c>
       <c r="B63" t="s">
-        <v>234</v>
+        <v>216</v>
       </c>
       <c r="C63" t="s">
-        <v>235</v>
+        <v>217</v>
       </c>
       <c r="D63" t="s">
-        <v>290</v>
+        <v>72</v>
       </c>
       <c r="E63" t="s">
-        <v>191</v>
+        <v>214</v>
       </c>
       <c r="F63" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G63">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H63">
         <v>1934</v>
@@ -3947,137 +4007,454 @@
         <v>1934</v>
       </c>
       <c r="J63" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K63">
+        <v>-84.085564000000005</v>
+      </c>
+      <c r="L63">
+        <v>9.9354469999999999</v>
       </c>
       <c r="M63" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T63" t="s">
-        <v>236</v>
+        <v>279</v>
       </c>
       <c r="U63" t="s">
-        <v>237</v>
+        <v>206</v>
       </c>
       <c r="X63" t="s">
         <v>114</v>
       </c>
       <c r="Y63">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="64" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>196</v>
+        <v>218</v>
       </c>
       <c r="B64" t="s">
-        <v>197</v>
+        <v>219</v>
       </c>
       <c r="C64" t="s">
-        <v>198</v>
+        <v>220</v>
       </c>
       <c r="D64" t="s">
-        <v>72</v>
+        <v>270</v>
       </c>
       <c r="E64" t="s">
-        <v>73</v>
+        <v>106</v>
+      </c>
+      <c r="F64" t="s">
+        <v>135</v>
+      </c>
+      <c r="G64">
+        <v>13</v>
       </c>
       <c r="H64">
-        <v>1928</v>
+        <v>1934</v>
       </c>
       <c r="I64">
-        <v>1928</v>
+        <v>1934</v>
       </c>
       <c r="J64" t="b">
-        <v>1</v>
-      </c>
-      <c r="K64">
-        <v>-74.247649999999993</v>
-      </c>
-      <c r="L64">
-        <v>11.00703</v>
+        <v>0</v>
       </c>
       <c r="M64" t="s">
-        <v>199</v>
+        <v>162</v>
+      </c>
+      <c r="N64" t="s">
+        <v>202</v>
+      </c>
+      <c r="O64" t="s">
+        <v>48</v>
+      </c>
+      <c r="P64" t="b">
+        <v>1</v>
       </c>
       <c r="T64" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+        <v>280</v>
+      </c>
+      <c r="U64" t="s">
+        <v>281</v>
+      </c>
+      <c r="X64" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y64">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="65" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>201</v>
+        <v>286</v>
       </c>
       <c r="B65" t="s">
-        <v>202</v>
+        <v>221</v>
       </c>
       <c r="C65" t="s">
-        <v>205</v>
+        <v>222</v>
       </c>
       <c r="D65" t="s">
         <v>72</v>
       </c>
       <c r="E65" t="s">
-        <v>73</v>
+        <v>289</v>
+      </c>
+      <c r="F65" t="s">
+        <v>135</v>
+      </c>
+      <c r="G65">
+        <v>14</v>
       </c>
       <c r="H65">
-        <v>1960</v>
+        <v>1934</v>
       </c>
       <c r="I65">
-        <v>1960</v>
+        <v>1934</v>
       </c>
       <c r="J65" t="b">
         <v>1</v>
       </c>
       <c r="K65">
-        <v>-79.680000000000007</v>
+        <v>-83.355490700000004</v>
       </c>
       <c r="L65">
-        <v>9.08</v>
+        <v>10.0877643</v>
       </c>
       <c r="M65" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+      <c r="Q65" t="s">
+        <v>135</v>
+      </c>
+      <c r="R65" t="s">
+        <v>76</v>
+      </c>
+      <c r="S65" t="b">
+        <v>1</v>
+      </c>
+      <c r="T65" t="s">
+        <v>223</v>
+      </c>
+      <c r="U65" t="s">
+        <v>224</v>
+      </c>
+      <c r="X65" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y65">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="66" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>204</v>
+        <v>292</v>
       </c>
       <c r="B66" t="s">
-        <v>203</v>
+        <v>287</v>
       </c>
       <c r="C66" t="s">
-        <v>206</v>
+        <v>288</v>
       </c>
       <c r="D66" t="s">
         <v>72</v>
       </c>
       <c r="E66" t="s">
+        <v>289</v>
+      </c>
+      <c r="F66" t="s">
+        <v>135</v>
+      </c>
+      <c r="G66">
+        <v>15</v>
+      </c>
+      <c r="H66">
+        <v>1934</v>
+      </c>
+      <c r="I66">
+        <v>1934</v>
+      </c>
+      <c r="J66" t="b">
+        <v>1</v>
+      </c>
+      <c r="K66">
+        <v>-83.355490700000004</v>
+      </c>
+      <c r="L66">
+        <v>10.0877643</v>
+      </c>
+      <c r="M66" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q66" t="s">
+        <v>104</v>
+      </c>
+      <c r="R66" t="s">
+        <v>290</v>
+      </c>
+      <c r="S66" t="b">
+        <v>1</v>
+      </c>
+      <c r="T66" t="s">
+        <v>293</v>
+      </c>
+      <c r="U66" t="s">
+        <v>294</v>
+      </c>
+      <c r="X66" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y66">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="67" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>298</v>
+      </c>
+      <c r="B67" t="s">
+        <v>296</v>
+      </c>
+      <c r="C67" t="s">
+        <v>297</v>
+      </c>
+      <c r="D67" t="s">
+        <v>270</v>
+      </c>
+      <c r="E67" t="s">
+        <v>250</v>
+      </c>
+      <c r="F67" t="s">
+        <v>135</v>
+      </c>
+      <c r="G67">
+        <v>16</v>
+      </c>
+      <c r="H67">
+        <v>1934</v>
+      </c>
+      <c r="I67">
+        <v>1934</v>
+      </c>
+      <c r="J67" t="b">
+        <v>0</v>
+      </c>
+      <c r="M67" t="s">
+        <v>162</v>
+      </c>
+      <c r="N67" t="s">
+        <v>48</v>
+      </c>
+      <c r="O67" t="s">
+        <v>58</v>
+      </c>
+      <c r="P67" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q67" t="s">
+        <v>104</v>
+      </c>
+      <c r="R67" t="s">
+        <v>58</v>
+      </c>
+      <c r="S67" t="b">
+        <v>1</v>
+      </c>
+      <c r="T67" t="s">
+        <v>299</v>
+      </c>
+      <c r="U67" t="s">
+        <v>300</v>
+      </c>
+      <c r="X67" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y67">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="68" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>301</v>
+      </c>
+      <c r="B68" t="s">
+        <v>302</v>
+      </c>
+      <c r="C68" t="s">
+        <v>303</v>
+      </c>
+      <c r="D68" t="s">
+        <v>270</v>
+      </c>
+      <c r="E68" t="s">
+        <v>250</v>
+      </c>
+      <c r="F68" t="s">
+        <v>135</v>
+      </c>
+      <c r="G68">
+        <v>16</v>
+      </c>
+      <c r="H68">
+        <v>1934</v>
+      </c>
+      <c r="I68">
+        <v>1934</v>
+      </c>
+      <c r="J68" t="b">
+        <v>0</v>
+      </c>
+      <c r="M68" t="s">
+        <v>162</v>
+      </c>
+      <c r="N68" t="s">
+        <v>48</v>
+      </c>
+      <c r="O68" t="s">
+        <v>284</v>
+      </c>
+      <c r="P68" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>290</v>
+      </c>
+      <c r="R68" t="s">
+        <v>284</v>
+      </c>
+      <c r="S68" t="b">
+        <v>1</v>
+      </c>
+      <c r="T68" t="s">
+        <v>304</v>
+      </c>
+      <c r="U68" t="s">
+        <v>305</v>
+      </c>
+      <c r="X68" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y68">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="69" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>190</v>
+      </c>
+      <c r="B69" t="s">
+        <v>191</v>
+      </c>
+      <c r="C69" t="s">
+        <v>192</v>
+      </c>
+      <c r="D69" t="s">
+        <v>72</v>
+      </c>
+      <c r="E69" t="s">
         <v>73</v>
       </c>
-      <c r="H66">
+      <c r="H69">
+        <v>1928</v>
+      </c>
+      <c r="I69">
+        <v>1928</v>
+      </c>
+      <c r="J69" t="b">
+        <v>1</v>
+      </c>
+      <c r="K69">
+        <v>-74.247649999999993</v>
+      </c>
+      <c r="L69">
+        <v>11.00703</v>
+      </c>
+      <c r="M69" t="s">
+        <v>193</v>
+      </c>
+      <c r="T69" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="70" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>195</v>
+      </c>
+      <c r="B70" t="s">
+        <v>196</v>
+      </c>
+      <c r="C70" t="s">
+        <v>199</v>
+      </c>
+      <c r="D70" t="s">
+        <v>72</v>
+      </c>
+      <c r="E70" t="s">
+        <v>73</v>
+      </c>
+      <c r="H70">
+        <v>1960</v>
+      </c>
+      <c r="I70">
+        <v>1960</v>
+      </c>
+      <c r="J70" t="b">
+        <v>1</v>
+      </c>
+      <c r="K70">
+        <v>-79.680000000000007</v>
+      </c>
+      <c r="L70">
+        <v>9.08</v>
+      </c>
+      <c r="M70" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="71" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>198</v>
+      </c>
+      <c r="B71" t="s">
+        <v>197</v>
+      </c>
+      <c r="C71" t="s">
+        <v>200</v>
+      </c>
+      <c r="D71" t="s">
+        <v>72</v>
+      </c>
+      <c r="E71" t="s">
+        <v>73</v>
+      </c>
+      <c r="H71">
         <v>1964</v>
       </c>
-      <c r="I66">
+      <c r="I71">
         <v>1964</v>
       </c>
-      <c r="J66" t="b">
-        <v>1</v>
-      </c>
-      <c r="K66">
+      <c r="J71" t="b">
+        <v>1</v>
+      </c>
+      <c r="K71">
         <v>-82.86206</v>
       </c>
-      <c r="L66">
+      <c r="L71">
         <v>8.2777499999999993</v>
       </c>
-      <c r="M66" t="s">
-        <v>207</v>
+      <c r="M71" t="s">
+        <v>201</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Minor fixes in data and legend.
* Updated legend.js so that the 'railroad' entry is displayed as a line with tick marks rather than a marker.
* Updated nodes.csv to improve spatial and temporal accuracy of some events in the Banana Strike of 1934 sequence, and standardized the use of the following terms: Banana Strike of 1934, Atlantic region, and UFCo.
* Improved writing in 1934_banana_strike.md.
* Added missing ES translation for 'movement.'
</commit_message>
<xml_diff>
--- a/data/nodes.xlsx
+++ b/data/nodes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro\Documents\GitHub\in-the-shadow-of-the-banana\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAEAA03-7BB0-45A6-A947-31A99F32C5A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BCDFE84-D6DB-4688-AD26-3E7916897D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5B9B3091-99AB-4305-BC97-7032E7BEE02C}"/>
   </bookViews>
@@ -497,9 +497,6 @@
     <t>Propiedad de Salomón Esna Miguel.</t>
   </si>
   <si>
-    <t>Finca más remota en la región Atlántica, junto al río Sixaola.</t>
-  </si>
-  <si>
     <t>Furthermost plantation in the Atlantic region of Costa Rica, next to the Sixaola River.</t>
   </si>
   <si>
@@ -510,15 +507,6 @@
   </si>
   <si>
     <t>Dueño de finca bananera.</t>
-  </si>
-  <si>
-    <t>Dueño de Finca Los Angeles.</t>
-  </si>
-  <si>
-    <t>Plantation owner of Los Angeles Plantation.</t>
-  </si>
-  <si>
-    <t>Manuel Mora recurre a su inmunidad legislativa para evadir el arresto y presentar recursos de habeas corpus en el Tribunal de Siquirres para liberar a los huelguistas arrestados durante la Huelga Bananera de 1934.</t>
   </si>
   <si>
     <t>Manuel Mora relies on his congressional immunity to avoid arrest and invoke habeas corpus in the Siquirres court to release workers arrested during the Banana Strike of 1934.</t>
@@ -703,33 +691,321 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">El Poder Ejecutivo, encabezado por el presidente Ricardo Jiménez Oreamuno, convocó una serie de reuniones consultivas en el </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Palacio Nacional</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> para mediar en la huelga bananera del Atlántico de 1934. Durante estas sesiones, la Presidencia interrogó a actores clave, incluido el finquero Arturo Volio. Tras la admisión de Volio sobre las condiciones laborales imperantes, el Ejecutivo atribuyó formalmente la responsabilidad del conflicto a las prácticas de gestión de las empresas bananeras.</t>
-    </r>
-  </si>
-  <si>
-    <t>Carlos Luis Fallas se trasladó desde la zona atlántica hasta San José para brindar testimonio ante el gobierno. Al comparecer en el Palacio Nacional, Fallas presentó un informe formal sobre las precarias condiciones de vida de los trabajadores, citando específicamente un salario diario de ₡4 y una tasa de incapacidad laboral del 50% debido a la malaria endémica.</t>
+    <t>fallas_deposition_1934</t>
+  </si>
+  <si>
+    <t>Workers Destroy Bananas</t>
+  </si>
+  <si>
+    <t>Police Cut and Gather Bananas</t>
+  </si>
+  <si>
+    <t>Arrest of Striking Workers</t>
+  </si>
+  <si>
+    <t>Habeas Corpus for Arrested Workers</t>
+  </si>
+  <si>
+    <t>mediation</t>
+  </si>
+  <si>
+    <t>Establecido como la sede principal del Estado costarricense, esta estructura neoclásica albergó el Poder Legislativo y las Secretarías de Estado (Poder Ejecutivo). Durante 103 años, funcionó como el núcleo administrativo centralizado del gobierno nacional hasta su demolición en 1958 para dar paso a la construcción del Banco Central de Costa Rica.</t>
+  </si>
+  <si>
+    <t>Executive Mediation of the 1934 Banana Strike</t>
+  </si>
+  <si>
+    <t>Mediación del Poder Ejecutivo en la huelga bananera de 1934</t>
+  </si>
+  <si>
+    <t>santos_inspection_1934</t>
+  </si>
+  <si>
+    <t>Ministerial Site Inspection of 26 Millas</t>
+  </si>
+  <si>
+    <t>Inspección ministerial en 26 Millas</t>
+  </si>
+  <si>
+    <t>Countermanded Order of Sabotage</t>
+  </si>
+  <si>
+    <t>Contraorden de sabotaje</t>
+  </si>
+  <si>
+    <t>Malaria Outbreak: Guápiles Sector</t>
+  </si>
+  <si>
+    <t>Brote de malaria: Sector Guápiles</t>
+  </si>
+  <si>
+    <t>migration</t>
+  </si>
+  <si>
+    <t>displacement</t>
+  </si>
+  <si>
+    <t>Sanitary Displacement: Guápiles to Siquirres</t>
+  </si>
+  <si>
+    <t>Desplazamiento sanitario: De Guápiles a Siquirres</t>
+  </si>
+  <si>
+    <t>Malaria Outbreak: Remote Plantations</t>
+  </si>
+  <si>
+    <t>Brote de malaria: Fincas remotas</t>
+  </si>
+  <si>
+    <t>Desplazamiento sanitario: Fincas remotas a Limón</t>
+  </si>
+  <si>
+    <t>Sanitary Displacement: Remote Plantations to Limón</t>
+  </si>
+  <si>
+    <t>Jaime Cerdas Mora reports a lack of medical infrastructure in the Guápiles sector. He notes that there were no resident doctors or local hospitals, leaving workers without immediate care during malaria outbreaks.</t>
+  </si>
+  <si>
+    <t>Jaime Cerdas Mora informa sobre la falta de infraestructura médica en el sector de Guápiles. Señala que no había médicos residentes ni hospitales locales, lo que dejaba a los trabajadores sin atención inmediata durante los brotes de malaria.</t>
+  </si>
+  <si>
+    <t>Jaime Cerdas Mora states that in remote plantations, malaria cases were frequent due to workers living in flooded barracks (ranchones). He estimates that half of the workers were unable to work half of the time because of the disease.</t>
+  </si>
+  <si>
+    <t>Cerdas describes workers from Guápiles traveling to Siquirres for treatment. He identifies the facility there as a dispensary staffed by a nurse rather than a doctor, where quinine was the only medicine provided.</t>
+  </si>
+  <si>
+    <t>Cerdas describe a los trabajadores de Guápiles viajando a Siquirres para recibir tratamiento. Identifica la instalación allí como un dispensario atendido por un enfermero en lugar de un médico, donde la quinina era el único medicamento suministrado.</t>
+  </si>
+  <si>
+    <t>Cerdas explains that workers in remote areas, such as those near the Sixaola river, were forced to travel to the city of Limón to find a hospital. This required sick laborers to travel long distances from the plantations to the provincial capital.</t>
+  </si>
+  <si>
+    <t>Cerdas explica que los trabajadores de zonas remotas, como las cercanas al río Sixaola, se veían obligados a trasladarse a la ciudad de Limón para encontrar un hospital. Esto requería que los obreros enfermos viajaran largas distancias desde las fincas hasta la capital provincial.</t>
+  </si>
+  <si>
+    <t>Judicial Confinement of Carlos Luis Fallas to Limón</t>
+  </si>
+  <si>
+    <t>Confinamiento judicial de Carlos Luis Fallas a Limón</t>
+  </si>
+  <si>
+    <t>declaration_strike_1934</t>
+  </si>
+  <si>
+    <t>demands_strike_1934</t>
+  </si>
+  <si>
+    <t>Leadership Deployment to 26 Millas</t>
+  </si>
+  <si>
+    <t>Despliegue de la dirigencia hacia 26 Millas</t>
+  </si>
+  <si>
+    <t>movement</t>
+  </si>
+  <si>
+    <t>comisariatos_1934_strike</t>
+  </si>
+  <si>
+    <t>Declaration of Strike</t>
+  </si>
+  <si>
+    <t>1934_strike_marker_003</t>
+  </si>
+  <si>
+    <t>worker_meeting_01_1934</t>
+  </si>
+  <si>
+    <t>87–88</t>
+  </si>
+  <si>
+    <t>Paralysis of the Atlantic Region</t>
+  </si>
+  <si>
+    <t>La paralización de la zona atlántica</t>
+  </si>
+  <si>
+    <t>Declaración de la huelga</t>
+  </si>
+  <si>
+    <t>Tras el rechazo del pliego de peticiones de los trabajadores por parte del gerente de la UFCo, George P. Chittenden. Los obreros sostuvieron una reunión cerca del 7 de agosto de 1934, en la que se acordó ir a huelga. Para entonces, ya se habían organizado comités de huelga en múltiples plantaciones, y Carlos Luis Fallas y Jaime Cerdas fueron encargados de dirigir el movimiento. Viajando en tren hasta Madre de Dios y luego a pie hacia 26 Millas, establecieron el principal cuartel operativo de la huelga cerca de la finca Los Ángeles. Según el relato de Cerdas, delegaciones de plantaciones a lo largo del corredor bananero atlántico ya se estaban reuniendo allí al momento de su llegada.</t>
+  </si>
+  <si>
+    <t>Deposition of Carlos Luis Fallas</t>
+  </si>
+  <si>
+    <t>Deposición de Carlos Luis Fallas</t>
+  </si>
+  <si>
+    <t>Presentación y rechazo del pliego de peticiones</t>
+  </si>
+  <si>
+    <t>Presentation and Rejection of the List of Demands</t>
+  </si>
+  <si>
+    <t>Cuartel general de los huelguistas durante la huelga bananera de 1934.</t>
+  </si>
+  <si>
+    <t>action</t>
+  </si>
+  <si>
+    <t>exploitation</t>
+  </si>
+  <si>
+    <t>public_site</t>
+  </si>
+  <si>
+    <t>deportation</t>
+  </si>
+  <si>
+    <t>Commissaries and the Scrip System</t>
+  </si>
+  <si>
+    <t>Los comisariatos y los cupones de la compañía</t>
+  </si>
+  <si>
+    <t>Following a strike organized in Alajuela, judicial authorities sentenced Carlos Luis Fallas to confinement in Limón, where he arrives in December 1933. This was a common legal penalty at the time, used to isolate political and labor leaders from their active organizational bases.</t>
+  </si>
+  <si>
+    <t>Tras una huelga que organizó en Alajuela, las autoridades judiciales sentenciaron a Carlos Luis Fallas a la pena de confinamiento en Limón, adonde llega en diciembre de 1933. Esta era una sanción legal común en la época, utilizada para aislar a líderes políticos y sindicales de sus bases organizativas activas.</t>
+  </si>
+  <si>
+    <t>The Minister of Government and Labor, Santos León Herrera, accompanied by the Chief of the Labor Section, Zayas Bazán, conducted a field inspection at the 26 Millas plantation during the absence of Carlos Luis Fallas. The visit functioned as a direct observation of the living quarters (ranchones), where the delegation encountered flooded dwellings and active cases of malaria.
+The event is noted for its impact on the Minister’s perspective. After witnessing the conditions and the confinement of workers, León Herrera explicitly conceded a divergence between "legality" and "justice."</t>
+  </si>
+  <si>
+    <t>El Ministro de Gobernación y Trabajo, Santos León Herrera, acompañado por el Jefe de la Sección de Trabajo, Zayas Bazán, realizó una inspección de campo en la finca 26 Millas durante la ausencia de Carlos Luis Fallas. La visita funcionó como una observación directa de los alojamientos (ranchones), donde la delegación constató viviendas inundadas y casos activos de malaria.
+El evento se destaca por su impacto en la perspectiva del Ministro. Tras presenciar las condiciones y el confinamiento de los trabajadores, León Herrera admitió explícitamente una divergencia entre lo "legal" y lo "justo".</t>
+  </si>
+  <si>
+    <t>Huelga bananera de 1934</t>
+  </si>
+  <si>
+    <t>Following the rejection of the workers’ petition by UFCo manager George P. Chittenden. Workers held a meeting around August 7, 1934 and agreed to go on strike. Strike committees had already been organized across multiple plantations, and Carlos Luis Fallas and Jaime Cerdas were tasked with directing the movement. Traveling by train to Madre de Dios and then on foot toward  26 Millas, they established the principal operational headquarters of the strike near the Los Ángeles plantation. According to Cerdas’ account, delegations from plantations across the Atlantic banana corridor were already gathering there upon their arrival.</t>
+  </si>
+  <si>
+    <t>finca_la_fortuna</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>countermanded_sabotage_1934</t>
+  </si>
+  <si>
+    <t>Conflict Between Fallas and Lino Bustos</t>
+  </si>
+  <si>
+    <t>Conflicto entre Fallas y Lino Bustos</t>
+  </si>
+  <si>
+    <t>confrontation</t>
+  </si>
+  <si>
+    <t>lino_bustos</t>
+  </si>
+  <si>
+    <t>Lino Bustos</t>
+  </si>
+  <si>
+    <t>fallas-bustos_conflict_1934</t>
+  </si>
+  <si>
+    <t>worker</t>
+  </si>
+  <si>
+    <t>Fallas Travels to Dos Bocas</t>
+  </si>
+  <si>
+    <t>Fallas viaja a Dos Bocas</t>
+  </si>
+  <si>
+    <t>fallas_to_dos_bocas_1934</t>
+  </si>
+  <si>
+    <t>bustos_to_la_fortuna_1934</t>
+  </si>
+  <si>
+    <t>Lino Bustos Sent to La Fortuna</t>
+  </si>
+  <si>
+    <t>Lino Bustos enviado a La Fortuna</t>
+  </si>
+  <si>
+    <t>Amid fears that the company might orchestrate acts of sabotage to discredit the strike movement, Jaime Cerdas received reports of possible threats at the plantation of La Fortuna. Taking advantage of the situation following Bustos’ conflict with Fallas, Cerdas assigned Lino Bustos to travel to La Fortuna and oversee the protection of company property and plantation operations in the area.</t>
+  </si>
+  <si>
+    <t>En medio de temores de que la compañía pudiera organizar actos de sabotaje para desacreditar al movimiento huelguístico, Jaime Cerdas recibió informes sobre posibles amenazas en la finca La Fortuna. Aprovechando la situación tras el conflicto entre Bustos y Fallas, Cerdas asignó a Lino Bustos la tarea de trasladarse a La Fortuna para supervisar la protección de la propiedad de la compañía y de las operaciones de la plantación en la zona.</t>
+  </si>
+  <si>
+    <t>company_town</t>
+  </si>
+  <si>
+    <t>As the 1934 banana strike expanded across the Atlantic zone, local authorities attempted to suppress the movement by ordering the arrest of striking workers traveling along public roads. According to Jaime Cerdas, these measures sought to disrupt communication and mobility between plantations participating in the strike.</t>
+  </si>
+  <si>
+    <t>Durante la huelga, Manuel Mora utilizó su inmunidad legislativa para evitar ser arrestado mientras operaba en Siquirres, donde presentó recursos de habeas corpus para obtener la liberación de trabajadores detenidos. Según Jaime Cerdas, la posición legal y política de Mora le permitió continuar coordinando apoyo para el movimiento a pesar de la represión gubernamental.</t>
+  </si>
+  <si>
+    <t>In response to the use of police labor, striking workers organized nighttime actions to destroy banana production near the plantations. According to Jaime Cerdas, workers overturned approximately ten hectares of banana fields, ensuring that no quality bananas reached Limón for export.</t>
+  </si>
+  <si>
+    <t>En respuesta al uso de fuerzas policiales como mano de obra, trabajadores huelguistas organizaron acciones nocturnas para destruir producción bananera cerca de las plantaciones. Según Jaime Cerdas, los trabajadores derribaron aproximadamente diez hectáreas de banano, asegurando que ningún banano de calidad llegara a Limón para su exportación.</t>
+  </si>
+  <si>
+    <t>violence</t>
+  </si>
+  <si>
+    <t>santos_leon_herrera</t>
+  </si>
+  <si>
+    <t>Santos León Herrera</t>
+  </si>
+  <si>
+    <t>official</t>
+  </si>
+  <si>
+    <t>Minister of Government and Labor (1932–1936)</t>
+  </si>
+  <si>
+    <t>Ministro de Gobernación y Trabajo (1932–1936)</t>
+  </si>
+  <si>
+    <t>In an effort to weaken the strike, authorities deployed police forces to cut and transport bananas in place of striking workers. The measure formed part of broader attempts by the government and the company to maintain banana production and contain the paralysis of the Atlantic region.</t>
+  </si>
+  <si>
+    <t>En un intento por debilitar la huelga, las autoridades desplegaron fuerzas policiales para cortar y transportar banano en sustitución de los trabajadores huelguistas. La medida formó parte de esfuerzos más amplios del gobierno y la compañía por mantener la producción bananera y contener la paralización de la región atlántica.</t>
+  </si>
+  <si>
+    <t>Manuel Mora recurre a su inmunidad legislativa para evadir el arresto y presentar recursos de habeas corpus en el Tribunal de Siquirres para liberar a los huelguistas arrestados durante la huelga bananera de 1934.</t>
+  </si>
+  <si>
+    <t>By the day following its formal declaration, the banana strike had spread across the Atlantic region. According to Jaime Cerdas, plantations throughout the region had already joined the movement, paralyzing production, transportation, and UFCo operations across the corridor.</t>
+  </si>
+  <si>
+    <t>Para el día siguiente de su declaración formal, la huelga bananera ya se había extendido por toda la región atlántica. Según Jaime Cerdas, plantaciones a lo largo de la región se habían incorporado al movimiento, paralizando la producción, el transporte y las operaciones de la UFCo en todo el corredor bananero.</t>
+  </si>
+  <si>
+    <t>On August 9, 1934, strike leaders formally declared the beginning of the banana strike. The declaration marked the transition from localized labor grievances to a coordinated regional movement across the Atlantic region.</t>
+  </si>
+  <si>
+    <t>El 9 de agosto de 1934, los dirigentes huelguistas declararon formalmente el inicio de la huelga bananera. La declaración marcó la transición de reclamos laborales localizados hacia un movimiento coordinado a escala regional en la región atlántica.</t>
+  </si>
+  <si>
+    <t>Based on the account by Jaime Cerdas Mora, the Communist Party drafted a formal list of demands and organized strike committees across the various banana plantations. The document was presented to the manager of UFCo, George P. Chittenden, who refused to receive it.</t>
+  </si>
+  <si>
+    <t>Según el relato de Jaime Cerdas Mora, el Partido Comunista redactó un pliego de peticiones formal y organizó comités de huelga en las diversas fincas bananeras. El documento fue presentado al gerente de la UFCo, George P. Chittenden, quien se negó a recibirlo.</t>
+  </si>
+  <si>
+    <t>UFCo and plantation-linked commissaries formed a system of economic dependency across the Atlantic region. Workers were frequently paid with coupons or tokens redeemable only at plantation commissaries, where goods were sold at inflated prices. According to Jaime Cerdas, this arrangement compounded already poor wages and living conditions, reinforcing what he described as a “double exploitation” of banana workers through both labor and controlled consumption.</t>
+  </si>
+  <si>
+    <t>Los comisariatos vinculados a la UFCo y a las fincas bananeras formaban un sistema de dependencia económica a lo largo de la región atlántica. Con frecuencia, los trabajadores eran pagados mediante cupones o chapas que solo podían utilizarse en los comisariatos de las plantaciones, donde los productos se vendían a precios elevados. Según el relato de Jaime Cerdas, este sistema agravaba los bajos salarios y las malas condiciones de vida, produciendo una “doble explotación” de los trabajadores bananeros a través tanto del trabajo como del consumo controlado.</t>
+  </si>
+  <si>
+    <t>Jaime Cerdas Mora afirma que en fincas remotas, los casos de malaria eran frecuentes debido a que los trabajadores vivían en ranchones inundados. Estima que la mitad de los trabajadores no podía laborar la mitad del tiempo a causa de la enfermedad.</t>
   </si>
   <si>
     <r>
@@ -775,218 +1051,64 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> labor incapacity rate due to endemic malaria.</t>
+      <t xml:space="preserve"> labor incapacity rate due to endemic malaria. During these sessions, the Presidency interrogated key stakeholders, including plantation owner Arturo Volio. Upon Volio’s admission of the prevailing labor conditions, President Jiménez attributed responsibility for the conflict to the banana industry's management practices.</t>
     </r>
   </si>
   <si>
-    <t>fallas_deposition_1934</t>
-  </si>
-  <si>
-    <t>Workers Destroy Bananas</t>
-  </si>
-  <si>
-    <t>Police Cut and Gather Bananas</t>
-  </si>
-  <si>
-    <t>Arrest of Striking Workers</t>
-  </si>
-  <si>
-    <t>Habeas Corpus for Arrested Workers</t>
-  </si>
-  <si>
-    <t>mediation</t>
-  </si>
-  <si>
-    <t>Establecido como la sede principal del Estado costarricense, esta estructura neoclásica albergó el Poder Legislativo y las Secretarías de Estado (Poder Ejecutivo). Durante 103 años, funcionó como el núcleo administrativo centralizado del gobierno nacional hasta su demolición en 1958 para dar paso a la construcción del Banco Central de Costa Rica.</t>
-  </si>
-  <si>
-    <t>Executive Mediation of the 1934 Banana Strike</t>
-  </si>
-  <si>
-    <t>Mediación del Poder Ejecutivo en la huelga bananera de 1934</t>
-  </si>
-  <si>
-    <t>santos_inspection_1934</t>
-  </si>
-  <si>
-    <t>Ministerial Site Inspection of 26 Millas</t>
-  </si>
-  <si>
-    <t>Inspección ministerial en 26 Millas</t>
-  </si>
-  <si>
-    <t>Countermanded Order of Sabotage</t>
-  </si>
-  <si>
-    <t>Contraorden de sabotaje</t>
-  </si>
-  <si>
-    <t>During a period of heightened tension in the 1934 strike, Carlos Luis Fallas—acting on unverified intelligence regarding approaching authorities—issued a written order to destroy a bridge to impede troop movement. Jaime Cerdas, co-leader of the movement, disputed the decision and unilaterally issued a countermand, nullifying the sabotage order without Fallas's immediate knowledge.</t>
-  </si>
-  <si>
-    <t>Durante un periodo de alta tensión en la huelga de 1934, Carlos Luis Fallas—actuando bajo inteligencia no verificada sobre el avance de las autoridades—emitió una orden escrita para destruir un puente y así impedir el movimiento de tropas. Jaime Cerdas, codirigente del movimiento, cuestionó la decisión y emitió unilateralmente una contraorden, anulando el sabotaje sin el conocimiento inmediato de Fallas.</t>
-  </si>
-  <si>
-    <t>Malaria Outbreak: Guápiles Sector</t>
-  </si>
-  <si>
-    <t>Brote de malaria: Sector Guápiles</t>
-  </si>
-  <si>
-    <t>migration</t>
-  </si>
-  <si>
-    <t>displacement</t>
-  </si>
-  <si>
-    <t>Sanitary Displacement: Guápiles to Siquirres</t>
-  </si>
-  <si>
-    <t>Desplazamiento sanitario: De Guápiles a Siquirres</t>
-  </si>
-  <si>
-    <t>Malaria Outbreak: Remote Plantations</t>
-  </si>
-  <si>
-    <t>Brote de malaria: Fincas remotas</t>
-  </si>
-  <si>
-    <t>Desplazamiento sanitario: Fincas remotas a Limón</t>
-  </si>
-  <si>
-    <t>Sanitary Displacement: Remote Plantations to Limón</t>
-  </si>
-  <si>
-    <t>Jaime Cerdas Mora reports a lack of medical infrastructure in the Guápiles sector. He notes that there were no resident doctors or local hospitals, leaving workers without immediate care during malaria outbreaks.</t>
-  </si>
-  <si>
-    <t>Jaime Cerdas Mora informa sobre la falta de infraestructura médica en el sector de Guápiles. Señala que no había médicos residentes ni hospitales locales, lo que dejaba a los trabajadores sin atención inmediata durante los brotes de malaria.</t>
-  </si>
-  <si>
-    <t>Jaime Cerdas Mora states that in remote plantations, malaria cases were frequent due to workers living in flooded barracks (ranchones). He estimates that half of the workers were unable to work half of the time because of the disease.</t>
-  </si>
-  <si>
-    <t>Jaime Cerdas Mora afirma que en fincas remotas, los casos de malaria eran frecuentes debido a que los trabajadores vivían en barracones (ranchones) inundados. Estima que la mitad de los trabajadores no podía laborar la mitad del tiempo a causa de la enfermedad.</t>
-  </si>
-  <si>
-    <t>Cerdas describes workers from Guápiles traveling to Siquirres for treatment. He identifies the facility there as a dispensary staffed by a nurse rather than a doctor, where quinine was the only medicine provided.</t>
-  </si>
-  <si>
-    <t>Cerdas describe a los trabajadores de Guápiles viajando a Siquirres para recibir tratamiento. Identifica la instalación allí como un dispensario atendido por un enfermero en lugar de un médico, donde la quinina era el único medicamento suministrado.</t>
-  </si>
-  <si>
-    <t>Cerdas explains that workers in remote areas, such as those near the Sixaola river, were forced to travel to the city of Limón to find a hospital. This required sick laborers to travel long distances from the plantations to the provincial capital.</t>
-  </si>
-  <si>
-    <t>Cerdas explica que los trabajadores de zonas remotas, como las cercanas al río Sixaola, se veían obligados a trasladarse a la ciudad de Limón para encontrar un hospital. Esto requería que los obreros enfermos viajaran largas distancias desde las fincas hasta la capital provincial.</t>
-  </si>
-  <si>
-    <t>Judicial Confinement of Carlos Luis Fallas to Limón</t>
-  </si>
-  <si>
-    <t>Confinamiento judicial de Carlos Luis Fallas a Limón</t>
-  </si>
-  <si>
-    <t>declaration_strike_1934</t>
-  </si>
-  <si>
-    <t>demands_strike_1934</t>
-  </si>
-  <si>
-    <t>Según el relato de Jaime Cerdas Mora, el Partido Comunista redactó un pliego de peticiones formal y organizó comités de huelga en las diversas fincas bananeras. El documento fue presentado al gerente de la United Fruit Company, George P. Chittenden, quien se negó a recibirlo.</t>
-  </si>
-  <si>
-    <t>Leadership Deployment to 26 Millas</t>
-  </si>
-  <si>
-    <t>Despliegue de la dirigencia hacia 26 Millas</t>
-  </si>
-  <si>
-    <t>movement</t>
-  </si>
-  <si>
-    <t>comisariatos_1934_strike</t>
-  </si>
-  <si>
-    <t>Los comisariatos vinculados a la UFCo y a las fincas bananeras formaban un sistema de dependencia económica a lo largo de la zona bananera atlántica. Con frecuencia, los trabajadores eran pagados mediante cupones o chapas que solo podían utilizarse en los comisariatos de las plantaciones, donde los productos se vendían a precios elevados. Según el relato de Jaime Cerdas, este sistema agravaba los bajos salarios y las malas condiciones de vida, produciendo una “doble explotación” de los trabajadores bananeros a través tanto del trabajo como del consumo controlado.</t>
-  </si>
-  <si>
-    <t>Declaration of Strike</t>
-  </si>
-  <si>
-    <t>1934_strike_marker_003</t>
-  </si>
-  <si>
-    <t>worker_meeting_01_1934</t>
-  </si>
-  <si>
-    <t>87–88</t>
-  </si>
-  <si>
-    <t>Paralysis of the Atlantic Region</t>
-  </si>
-  <si>
-    <t>La paralización de la zona atlántica</t>
-  </si>
-  <si>
-    <t>Declaración de la huelga</t>
-  </si>
-  <si>
-    <t>By the day following its formal declaration, the 1934 banana strike had spread across the Atlantic banana zone. According to Jaime Cerdas, plantations throughout the region had already joined the movement, paralyzing production, transportation, and UFCo operations across the corridor.</t>
-  </si>
-  <si>
-    <t>Para el día siguiente de su declaración formal, la huelga bananera de 1934 ya se había extendido por toda la zona bananera atlántica. Según Jaime Cerdas, plantaciones a lo largo de la región se habían incorporado al movimiento, paralizando la producción, el transporte y las operaciones de la UFCo en todo el corredor bananero.</t>
-  </si>
-  <si>
-    <t>Tras el rechazo del pliego de peticiones de los trabajadores por parte del gerente de la UFCo, George P. Chittenden. Los obreros sostuvieron una reunión cerca del 7 de agosto de 1934, en la que se acordó ir a huelga. Para entonces, ya se habían organizado comités de huelga en múltiples plantaciones, y Carlos Luis Fallas y Jaime Cerdas fueron encargados de dirigir el movimiento. Viajando en tren hasta Madre de Dios y luego a pie hacia 26 Millas, establecieron el principal cuartel operativo de la huelga cerca de la finca Los Ángeles. Según el relato de Cerdas, delegaciones de plantaciones a lo largo del corredor bananero atlántico ya se estaban reuniendo allí al momento de su llegada.</t>
-  </si>
-  <si>
-    <t>On August 9, 1934, strike leaders formally declared the beginning of the banana strike. The declaration marked the transition from localized labor grievances to a coordinated regional movement across the Atlantic banana zone.</t>
-  </si>
-  <si>
-    <t>El 9 de agosto de 1934, los dirigentes huelguistas declararon formalmente el inicio de la huelga bananera. La declaración marcó la transición de reclamos laborales localizados hacia un movimiento coordinado a escala regional en la zona bananera atlántica.</t>
-  </si>
-  <si>
-    <t>Deposition of Carlos Luis Fallas</t>
-  </si>
-  <si>
-    <t>Deposición de Carlos Luis Fallas</t>
-  </si>
-  <si>
-    <t>Presentación y rechazo del pliego de peticiones</t>
-  </si>
-  <si>
-    <t>Presentation and Rejection of the List of Demands</t>
-  </si>
-  <si>
-    <t>Cuartel general de los huelguistas durante la huelga bananera de 1934.</t>
-  </si>
-  <si>
-    <t>action</t>
-  </si>
-  <si>
-    <t>exploitation</t>
-  </si>
-  <si>
-    <t>public_site</t>
-  </si>
-  <si>
-    <t>deportation</t>
-  </si>
-  <si>
-    <t>Commissaries and the Scrip System</t>
-  </si>
-  <si>
-    <t>Los comisariatos y los cupones de la compañía</t>
-  </si>
-  <si>
-    <t>UFCo and plantation-linked commissaries formed a system of economic dependency across the Atlantic banana zone. Workers were frequently paid with coupons or tokens redeemable only at plantation commissaries, where goods were sold at inflated prices. According to Jaime Cerdas, this arrangement compounded already poor wages and living conditions, reinforcing what he described as a “double exploitation” of banana workers through both labor and controlled consumption.</t>
-  </si>
-  <si>
-    <t>Following a strike organized in Alajuela, judicial authorities sentenced Carlos Luis Fallas to confinement in Limón, where he arrives in December 1933. This was a common legal penalty at the time, used to isolate political and labor leaders from their active organizational bases.</t>
-  </si>
-  <si>
-    <t>Tras una huelga que organizó en Alajuela, las autoridades judiciales sentenciaron a Carlos Luis Fallas a la pena de confinamiento en Limón, adonde llega en diciembre de 1933. Esta era una sanción legal común en la época, utilizada para aislar a líderes políticos y sindicales de sus bases organizativas activas.</t>
+    <t>Carlos Luis Fallas se trasladó desde la zona atlántica hasta San José para brindar testimonio ante el gobierno. Al comparecer en el Palacio Nacional, Fallas presentó un informe formal sobre las precarias condiciones de vida de los trabajadores, citando específicamente un salario diario de ₡4 y una tasa de incapacidad laboral del 50% debido a la malaria endémica. Durante estas sesiones, la Presidencia interrogó a actores clave, incluido el finquero Arturo Volio. Tras la admisión de Volio sobre las condiciones laborales imperantes, el presidente Jiménez atribuyó la responsabilidad del conflicto a las prácticas de gestión de las empresas bananeras.</t>
+  </si>
+  <si>
+    <t>Dueño de la finca Los Angeles.</t>
+  </si>
+  <si>
+    <t>Owner of Los Angeles plantation.</t>
+  </si>
+  <si>
+    <t>Finca más remota en la región Atlántica de Costa Rica, junto al río Sixaola.</t>
+  </si>
+  <si>
+    <t>Tras la confrontación con Lino Bustos, Carlos Luis Fallas partió hacia Dos Bocas mientras continuaban los esfuerzos de coordinación de la huelga en la región atlántica. Su desplazamiento formó parte de la actividad organizativa más amplia mediante la cual los dirigentes huelguísticos se movilizaban entre plantaciones y campamentos para mantener la comunicación y la dirección del movimiento.</t>
+  </si>
+  <si>
+    <t>Following the confrontation with Lino Bustos, Carlos Luis Fallas departed for Dos Bocas while strike coordination efforts continued across the Atlantic region. His movement formed part of the broader organizational activity through which strike leaders traveled between plantations and camps to maintain communication and direction during the conflict.</t>
+  </si>
+  <si>
+    <t>During the banana strike, tensions emerged within the strike movement itself when Carlos Luis Fallas became involved in a heated confrontation with a worker named Lino Bustos, described by Jaime Cerdas as an admirer of Fallas. According to Cerdas, the argument escalated to the point that Bustos drew a knife and began threatening Fallas before the situation dissipated. The incident illustrates the internal pressures and personal conflicts that developed within the rapidly expanding strike movement.</t>
+  </si>
+  <si>
+    <t>Durante la huelga bananera, surgieron tensiones dentro del propio movimiento huelguístico cuando Carlos Luis Fallas se vio involucrado en una fuerte confrontación con un trabajador llamado Lino Bustos, descrito por Jaime Cerdas como admirador de Fallas. Según Cerdas, la discusión escaló hasta el punto en que Bustos sacó un cuchillo y comenzó a amenazar a Fallas antes de que la situación se disipara. El incidente refleja las presiones internas y los conflictos personales que surgieron dentro del movimiento huelguístico en rápida expansión.</t>
+  </si>
+  <si>
+    <t>During a period of heightened tension in the strike, Carlos Luis Fallas—acting on unverified intelligence regarding approaching authorities—issued a written order to destroy a bridge to impede troop movement. Jaime Cerdas, co-leader of the movement, disputed the decision and unilaterally issued a countermand, nullifying the sabotage order without Fallas's immediate knowledge.</t>
+  </si>
+  <si>
+    <t>Durante un periodo de alta tensión en la huelga, Carlos Luis Fallas—actuando bajo inteligencia no verificada sobre el avance de las autoridades—emitió una orden escrita para destruir un puente y así impedir el movimiento de tropas. Jaime Cerdas, codirigente del movimiento, cuestionó la decisión y emitió unilateralmente una contraorden, anulando el sabotaje sin el conocimiento inmediato de Fallas.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">El Poder Ejecutivo, encabezado por el presidente Ricardo Jiménez Oreamuno, convocó una serie de reuniones consultivas en el </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Palacio Nacional</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> para mediar en la huelga bananera.</t>
+    </r>
   </si>
   <si>
     <r>
@@ -1011,130 +1133,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> to mediate the 1934 banana strike. During these sessions, the Presidency interrogated key stakeholders, including plantation owner Arturo Volio. Upon Volio’s admission of the prevailing labor conditions, the Executive formally attributed responsibility for the conflict to the banana industry's management practices.</t>
+      <t xml:space="preserve"> to mediate the banana strike.</t>
     </r>
-  </si>
-  <si>
-    <t>The Minister of Government and Labor, Santos León Herrera, accompanied by the Chief of the Labor Section, Zayas Bazán, conducted a field inspection at the 26 Millas plantation during the absence of Carlos Luis Fallas. The visit functioned as a direct observation of the living quarters (ranchones), where the delegation encountered flooded dwellings and active cases of malaria.
-The event is noted for its impact on the Minister’s perspective. After witnessing the conditions and the confinement of workers, León Herrera explicitly conceded a divergence between "legality" and "justice."</t>
-  </si>
-  <si>
-    <t>El Ministro de Gobernación y Trabajo, Santos León Herrera, acompañado por el Jefe de la Sección de Trabajo, Zayas Bazán, realizó una inspección de campo en la finca 26 Millas durante la ausencia de Carlos Luis Fallas. La visita funcionó como una observación directa de los alojamientos (ranchones), donde la delegación constató viviendas inundadas y casos activos de malaria.
-El evento se destaca por su impacto en la perspectiva del Ministro. Tras presenciar las condiciones y el confinamiento de los trabajadores, León Herrera admitió explícitamente una divergencia entre lo "legal" y lo "justo".</t>
-  </si>
-  <si>
-    <t>Huelga bananera de 1934</t>
-  </si>
-  <si>
-    <t>Following the rejection of the workers’ petition by UFCo manager George P. Chittenden. Workers held a meeting around August 7, 1934 and agreed to go on strike. Strike committees had already been organized across multiple plantations, and Carlos Luis Fallas and Jaime Cerdas were tasked with directing the movement. Traveling by train to Madre de Dios and then on foot toward  26 Millas, they established the principal operational headquarters of the strike near the Los Ángeles plantation. According to Cerdas’ account, delegations from plantations across the Atlantic banana corridor were already gathering there upon their arrival.</t>
-  </si>
-  <si>
-    <t>finca_la_fortuna</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>countermanded_sabotage_1934</t>
-  </si>
-  <si>
-    <t>Conflict Between Fallas and Lino Bustos</t>
-  </si>
-  <si>
-    <t>Conflicto entre Fallas y Lino Bustos</t>
-  </si>
-  <si>
-    <t>confrontation</t>
-  </si>
-  <si>
-    <t>lino_bustos</t>
-  </si>
-  <si>
-    <t>Lino Bustos</t>
-  </si>
-  <si>
-    <t>fallas-bustos_conflict_1934</t>
-  </si>
-  <si>
-    <t>During the 1934 banana strike, tensions emerged within the strike movement itself when Carlos Luis Fallas became involved in a heated confrontation with a worker named Lino Bustos, described by Jaime Cerdas as an admirer of Fallas. According to Cerdas, the argument escalated to the point that Bustos drew a knife and began threatening Fallas before the situation dissipated. The incident illustrates the internal pressures and personal conflicts that developed within the rapidly expanding strike movement.</t>
-  </si>
-  <si>
-    <t>Durante la huelga bananera de 1934, surgieron tensiones dentro del propio movimiento huelguístico cuando Carlos Luis Fallas se vio involucrado en una fuerte confrontación con un trabajador llamado Lino Bustos, descrito por Jaime Cerdas como admirador de Fallas. Según Cerdas, la discusión escaló hasta el punto en que Bustos sacó un cuchillo y comenzó a amenazar a Fallas antes de que la situación se disipara. El incidente refleja las presiones internas y los conflictos personales que surgieron dentro del movimiento huelguístico en rápida expansión.</t>
-  </si>
-  <si>
-    <t>worker</t>
-  </si>
-  <si>
-    <t>Fallas Travels to Dos Bocas</t>
-  </si>
-  <si>
-    <t>Fallas viaja a Dos Bocas</t>
-  </si>
-  <si>
-    <t>fallas_to_dos_bocas_1934</t>
-  </si>
-  <si>
-    <t>Following the confrontation with Lino Bustos, Carlos Luis Fallas departed for Dos Bocas while strike coordination efforts continued across the Atlantic banana zone. His movement formed part of the broader organizational activity through which strike leaders traveled between plantations and camps to maintain communication and direction during the conflict.</t>
-  </si>
-  <si>
-    <t>Tras la confrontación con Lino Bustos, Carlos Luis Fallas partió hacia Dos Bocas mientras continuaban los esfuerzos de coordinación de la huelga en la zona bananera atlántica. Su desplazamiento formó parte de la actividad organizativa más amplia mediante la cual los dirigentes huelguísticos se movilizaban entre plantaciones y campamentos para mantener la comunicación y la dirección del movimiento.</t>
-  </si>
-  <si>
-    <t>bustos_to_la_fortuna_1934</t>
-  </si>
-  <si>
-    <t>Lino Bustos Sent to La Fortuna</t>
-  </si>
-  <si>
-    <t>Lino Bustos enviado a La Fortuna</t>
-  </si>
-  <si>
-    <t>Amid fears that the company might orchestrate acts of sabotage to discredit the strike movement, Jaime Cerdas received reports of possible threats at the plantation of La Fortuna. Taking advantage of the situation following Bustos’ conflict with Fallas, Cerdas assigned Lino Bustos to travel to La Fortuna and oversee the protection of company property and plantation operations in the area.</t>
-  </si>
-  <si>
-    <t>En medio de temores de que la compañía pudiera organizar actos de sabotaje para desacreditar al movimiento huelguístico, Jaime Cerdas recibió informes sobre posibles amenazas en la finca La Fortuna. Aprovechando la situación tras el conflicto entre Bustos y Fallas, Cerdas asignó a Lino Bustos la tarea de trasladarse a La Fortuna para supervisar la protección de la propiedad de la compañía y de las operaciones de la plantación en la zona.</t>
-  </si>
-  <si>
-    <t>company_town</t>
-  </si>
-  <si>
-    <t>Based on the account by Jaime Cerdas Mora, the Communist Party drafted a formal list of demands and organized strike committees across the various banana plantations. The document was presented to the manager of the United Fruit Company, George P. Chittenden, who refused to receive it.</t>
-  </si>
-  <si>
-    <t>As the 1934 banana strike expanded across the Atlantic zone, local authorities attempted to suppress the movement by ordering the arrest of striking workers traveling along public roads. According to Jaime Cerdas, these measures sought to disrupt communication and mobility between plantations participating in the strike.</t>
-  </si>
-  <si>
-    <t>Durante la huelga, Manuel Mora utilizó su inmunidad legislativa para evitar ser arrestado mientras operaba en Siquirres, donde presentó recursos de habeas corpus para obtener la liberación de trabajadores detenidos. Según Jaime Cerdas, la posición legal y política de Mora le permitió continuar coordinando apoyo para el movimiento a pesar de la represión gubernamental.</t>
-  </si>
-  <si>
-    <t>In an effort to weaken the strike, authorities deployed police forces to cut and transport bananas in place of striking workers. The measure formed part of broader attempts by the government and the company to maintain banana production and contain the paralysis of the Atlantic banana zone.</t>
-  </si>
-  <si>
-    <t>En un intento por debilitar la huelga, las autoridades desplegaron fuerzas policiales para cortar y transportar banano en sustitución de los trabajadores huelguistas. La medida formó parte de esfuerzos más amplios del gobierno y la compañía por mantener la producción bananera y contener la paralización de la zona bananera atlántica.</t>
-  </si>
-  <si>
-    <t>In response to the use of police labor, striking workers organized nighttime actions to destroy banana production near the plantations. According to Jaime Cerdas, workers overturned approximately ten hectares of banana fields, ensuring that no quality bananas reached Limón for export.</t>
-  </si>
-  <si>
-    <t>En respuesta al uso de fuerzas policiales como mano de obra, trabajadores huelguistas organizaron acciones nocturnas para destruir producción bananera cerca de las plantaciones. Según Jaime Cerdas, los trabajadores derribaron aproximadamente diez hectáreas de banano, asegurando que ningún banano de calidad llegara a Limón para su exportación.</t>
-  </si>
-  <si>
-    <t>violence</t>
-  </si>
-  <si>
-    <t>santos_leon_herrera</t>
-  </si>
-  <si>
-    <t>Santos León Herrera</t>
-  </si>
-  <si>
-    <t>official</t>
-  </si>
-  <si>
-    <t>Minister of Government and Labor (1932–1936)</t>
-  </si>
-  <si>
-    <t>Ministro de Gobernación y Trabajo (1932–1936)</t>
   </si>
 </sst>
 </file>
@@ -1606,10 +1606,10 @@
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="G1" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="H1" t="s">
         <v>6</v>
@@ -1627,7 +1627,7 @@
         <v>5</v>
       </c>
       <c r="M1" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="N1" t="s">
         <v>8</v>
@@ -1657,7 +1657,7 @@
         <v>15</v>
       </c>
       <c r="W1" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="X1" t="s">
         <v>14</v>
@@ -1692,7 +1692,7 @@
         <v>9.9281000000000006</v>
       </c>
       <c r="M2" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
@@ -1721,7 +1721,7 @@
         <v>10.0162</v>
       </c>
       <c r="M3" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
@@ -1750,7 +1750,7 @@
         <v>9.9002999999999997</v>
       </c>
       <c r="M4" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
@@ -1779,7 +1779,7 @@
         <v>9.9922000000000004</v>
       </c>
       <c r="M5" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
@@ -1808,7 +1808,7 @@
         <v>9.9901999999999997</v>
       </c>
       <c r="M6" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
@@ -1837,7 +1837,7 @@
         <v>42.360100000000003</v>
       </c>
       <c r="M7" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
@@ -1866,7 +1866,7 @@
         <v>42.360300000000002</v>
       </c>
       <c r="M8" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
@@ -1895,7 +1895,7 @@
         <v>10.097</v>
       </c>
       <c r="M9" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
@@ -1924,7 +1924,7 @@
         <v>29.9499</v>
       </c>
       <c r="M10" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
@@ -1956,7 +1956,7 @@
         <v>10.050000000000001</v>
       </c>
       <c r="M11" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T11" t="s">
         <v>47</v>
@@ -1997,7 +1997,7 @@
         <v>10.02</v>
       </c>
       <c r="M12" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T12" t="s">
         <v>45</v>
@@ -2035,7 +2035,7 @@
         <v>10.08</v>
       </c>
       <c r="M13" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T13" t="s">
         <v>45</v>
@@ -2073,7 +2073,7 @@
         <v>10.1</v>
       </c>
       <c r="M14" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T14" t="s">
         <v>45</v>
@@ -2111,7 +2111,7 @@
         <v>9.9</v>
       </c>
       <c r="M15" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T15" t="s">
         <v>46</v>
@@ -2134,7 +2134,7 @@
         <v>24</v>
       </c>
       <c r="E16" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="H16">
         <v>1934</v>
@@ -2152,13 +2152,13 @@
         <v>10.0877643</v>
       </c>
       <c r="M16" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T16" t="s">
         <v>150</v>
       </c>
       <c r="U16" t="s">
-        <v>269</v>
+        <v>253</v>
       </c>
       <c r="X16" t="s">
         <v>114</v>
@@ -2187,7 +2187,7 @@
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T17" t="s">
         <v>71</v>
@@ -2225,7 +2225,7 @@
         <v>10.094110000000001</v>
       </c>
       <c r="M18" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="X18" t="s">
         <v>114</v>
@@ -2260,7 +2260,7 @@
         <v>10.215439999999999</v>
       </c>
       <c r="M19" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
@@ -2277,7 +2277,7 @@
         <v>24</v>
       </c>
       <c r="E20" t="s">
-        <v>306</v>
+        <v>284</v>
       </c>
       <c r="J20" t="b">
         <v>1</v>
@@ -2289,12 +2289,12 @@
         <v>10.28565</v>
       </c>
       <c r="M20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>284</v>
+        <v>266</v>
       </c>
       <c r="B21" t="s">
         <v>130</v>
@@ -2318,10 +2318,10 @@
         <v>9.7301959999999994</v>
       </c>
       <c r="M21" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N21" t="s">
-        <v>285</v>
+        <v>267</v>
       </c>
       <c r="X21" t="s">
         <v>114</v>
@@ -2356,7 +2356,7 @@
         <v>10.17947</v>
       </c>
       <c r="M22" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
@@ -2385,7 +2385,7 @@
         <v>10.086040000000001</v>
       </c>
       <c r="M23" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.25">
@@ -2414,7 +2414,7 @@
         <v>10.08187</v>
       </c>
       <c r="M24" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
@@ -2443,13 +2443,13 @@
         <v>9.5016700000000007</v>
       </c>
       <c r="M25" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T25" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="U25" t="s">
-        <v>152</v>
+        <v>311</v>
       </c>
       <c r="X25" t="s">
         <v>114</v>
@@ -2466,7 +2466,7 @@
         <v>136</v>
       </c>
       <c r="C26" t="s">
-        <v>282</v>
+        <v>264</v>
       </c>
       <c r="D26" t="s">
         <v>72</v>
@@ -2493,7 +2493,7 @@
         <v>10.0877643</v>
       </c>
       <c r="M26" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="V26" t="b">
         <v>1</v>
@@ -2582,19 +2582,19 @@
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B30" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C30" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D30" t="s">
         <v>25</v>
       </c>
       <c r="E30" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="H30">
         <v>1885</v>
@@ -2612,7 +2612,7 @@
         <v>-71.049722000000003</v>
       </c>
       <c r="M30" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
@@ -2635,7 +2635,7 @@
         <v>0</v>
       </c>
       <c r="M31" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
@@ -2658,7 +2658,7 @@
         <v>0</v>
       </c>
       <c r="M32" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.25">
@@ -2681,7 +2681,7 @@
         <v>0</v>
       </c>
       <c r="M33" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.25">
@@ -2704,7 +2704,7 @@
         <v>0</v>
       </c>
       <c r="M34" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.25">
@@ -2721,7 +2721,7 @@
         <v>74</v>
       </c>
       <c r="E35" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="H35">
         <v>1931</v>
@@ -2730,7 +2730,7 @@
         <v>0</v>
       </c>
       <c r="M35" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.25">
@@ -2744,19 +2744,19 @@
         <v>91</v>
       </c>
       <c r="D36" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E36" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="J36" t="b">
         <v>0</v>
       </c>
       <c r="T36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="U36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="V36" t="b">
         <v>1</v>
@@ -2773,10 +2773,10 @@
         <v>89</v>
       </c>
       <c r="D37" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E37" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="J37" t="b">
         <v>0</v>
@@ -2796,16 +2796,16 @@
         <v>94</v>
       </c>
       <c r="D38" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E38" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="J38" t="b">
         <v>0</v>
       </c>
       <c r="M38" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="39" spans="1:25" x14ac:dyDescent="0.25">
@@ -2819,16 +2819,16 @@
         <v>105</v>
       </c>
       <c r="D39" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E39" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="J39" t="b">
         <v>0</v>
       </c>
       <c r="M39" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.25">
@@ -2842,22 +2842,22 @@
         <v>96</v>
       </c>
       <c r="D40" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E40" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="J40" t="b">
         <v>0</v>
       </c>
       <c r="M40" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T40" t="s">
         <v>103</v>
       </c>
       <c r="U40" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="X40" t="s">
         <v>114</v>
@@ -2877,22 +2877,22 @@
         <v>98</v>
       </c>
       <c r="D41" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E41" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="J41" t="b">
         <v>0</v>
       </c>
       <c r="M41" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T41" t="s">
         <v>103</v>
       </c>
       <c r="U41" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="X41" t="s">
         <v>114</v>
@@ -2912,22 +2912,22 @@
         <v>100</v>
       </c>
       <c r="D42" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E42" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="J42" t="b">
         <v>0</v>
       </c>
       <c r="M42" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T42" t="s">
-        <v>158</v>
+        <v>310</v>
       </c>
       <c r="U42" t="s">
-        <v>157</v>
+        <v>309</v>
       </c>
       <c r="X42" t="s">
         <v>114</v>
@@ -2947,68 +2947,68 @@
         <v>102</v>
       </c>
       <c r="D43" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E43" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="J43" t="b">
         <v>0</v>
       </c>
       <c r="M43" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="44" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>315</v>
+        <v>290</v>
       </c>
       <c r="B44" t="s">
-        <v>316</v>
+        <v>291</v>
       </c>
       <c r="C44" t="s">
-        <v>316</v>
+        <v>291</v>
       </c>
       <c r="D44" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E44" t="s">
-        <v>317</v>
+        <v>292</v>
       </c>
       <c r="J44" t="b">
         <v>0</v>
       </c>
       <c r="M44" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T44" t="s">
-        <v>318</v>
+        <v>293</v>
       </c>
       <c r="U44" t="s">
-        <v>319</v>
+        <v>294</v>
       </c>
     </row>
     <row r="45" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>290</v>
+        <v>272</v>
       </c>
       <c r="B45" t="s">
-        <v>291</v>
+        <v>273</v>
       </c>
       <c r="C45" t="s">
-        <v>291</v>
+        <v>273</v>
       </c>
       <c r="D45" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E45" t="s">
-        <v>295</v>
+        <v>275</v>
       </c>
       <c r="J45" t="b">
         <v>0</v>
       </c>
       <c r="M45" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="46" spans="1:25" x14ac:dyDescent="0.25">
@@ -3025,7 +3025,7 @@
         <v>14</v>
       </c>
       <c r="E46" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="H46">
         <v>1984</v>
@@ -3043,7 +3043,7 @@
         <v>9.9281000000000006</v>
       </c>
       <c r="M46" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="V46" t="b">
         <v>1</v>
@@ -3063,16 +3063,16 @@
         <v>116</v>
       </c>
       <c r="B47" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="C47" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="D47" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="E47" t="s">
-        <v>273</v>
+        <v>257</v>
       </c>
       <c r="F47" t="s">
         <v>135</v>
@@ -3090,7 +3090,7 @@
         <v>0</v>
       </c>
       <c r="M47" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N47" t="s">
         <v>67</v>
@@ -3111,10 +3111,10 @@
         <v>1</v>
       </c>
       <c r="T47" t="s">
-        <v>277</v>
+        <v>260</v>
       </c>
       <c r="U47" t="s">
-        <v>278</v>
+        <v>261</v>
       </c>
       <c r="X47" t="s">
         <v>114</v>
@@ -3125,19 +3125,19 @@
     </row>
     <row r="48" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B48" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="C48" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="D48" t="s">
         <v>72</v>
       </c>
       <c r="E48" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F48" t="s">
         <v>135</v>
@@ -3161,13 +3161,13 @@
         <v>9.5500000000000007</v>
       </c>
       <c r="M48" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T48" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="U48" t="s">
-        <v>238</v>
+        <v>306</v>
       </c>
       <c r="X48" t="s">
         <v>114</v>
@@ -3178,19 +3178,19 @@
     </row>
     <row r="49" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B49" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C49" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="D49" t="s">
         <v>72</v>
       </c>
       <c r="E49" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F49" t="s">
         <v>135</v>
@@ -3214,13 +3214,13 @@
         <v>10.217700000000001</v>
       </c>
       <c r="M49" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T49" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="U49" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="X49" t="s">
         <v>114</v>
@@ -3231,19 +3231,19 @@
     </row>
     <row r="50" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B50" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="C50" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="D50" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="E50" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="F50" t="s">
         <v>135</v>
@@ -3261,10 +3261,10 @@
         <v>0</v>
       </c>
       <c r="M50" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N50" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="O50" t="s">
         <v>18</v>
@@ -3273,10 +3273,10 @@
         <v>1</v>
       </c>
       <c r="T50" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="U50" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="X50" t="s">
         <v>114</v>
@@ -3287,19 +3287,19 @@
     </row>
     <row r="51" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B51" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="C51" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="D51" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="E51" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="F51" t="s">
         <v>135</v>
@@ -3317,10 +3317,10 @@
         <v>0</v>
       </c>
       <c r="M51" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N51" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="O51" t="s">
         <v>27</v>
@@ -3329,10 +3329,10 @@
         <v>1</v>
       </c>
       <c r="T51" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="U51" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="X51" t="s">
         <v>114</v>
@@ -3343,19 +3343,19 @@
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="B52" t="s">
-        <v>274</v>
+        <v>258</v>
       </c>
       <c r="C52" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="D52" t="s">
         <v>72</v>
       </c>
       <c r="E52" t="s">
-        <v>271</v>
+        <v>255</v>
       </c>
       <c r="F52" t="s">
         <v>135</v>
@@ -3379,13 +3379,13 @@
         <v>10.097</v>
       </c>
       <c r="M52" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T52" t="s">
-        <v>276</v>
+        <v>304</v>
       </c>
       <c r="U52" t="s">
-        <v>252</v>
+        <v>305</v>
       </c>
       <c r="X52" t="s">
         <v>114</v>
@@ -3396,19 +3396,19 @@
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="B53" t="s">
-        <v>268</v>
+        <v>252</v>
       </c>
       <c r="C53" t="s">
-        <v>267</v>
+        <v>251</v>
       </c>
       <c r="D53" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E53" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="F53" t="s">
         <v>135</v>
@@ -3426,7 +3426,7 @@
         <v>0</v>
       </c>
       <c r="M53" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N53" t="s">
         <v>16</v>
@@ -3447,10 +3447,10 @@
         <v>1</v>
       </c>
       <c r="T53" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="U53" t="s">
-        <v>247</v>
+        <v>303</v>
       </c>
       <c r="X53" t="s">
         <v>114</v>
@@ -3461,19 +3461,19 @@
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="B54" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="C54" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="D54" t="s">
         <v>72</v>
       </c>
       <c r="E54" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="F54" t="s">
         <v>135</v>
@@ -3491,7 +3491,7 @@
         <v>0</v>
       </c>
       <c r="M54" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N54" t="s">
         <v>18</v>
@@ -3503,10 +3503,10 @@
         <v>1</v>
       </c>
       <c r="T54" t="s">
-        <v>283</v>
+        <v>265</v>
       </c>
       <c r="U54" t="s">
-        <v>262</v>
+        <v>248</v>
       </c>
       <c r="X54" t="s">
         <v>114</v>
@@ -3517,19 +3517,19 @@
     </row>
     <row r="55" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="B55" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="C55" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="D55" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E55" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="F55" t="s">
         <v>135</v>
@@ -3547,7 +3547,7 @@
         <v>1</v>
       </c>
       <c r="M55" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N55" t="s">
         <v>48</v>
@@ -3556,27 +3556,27 @@
         <v>17</v>
       </c>
       <c r="T55" t="s">
-        <v>263</v>
+        <v>300</v>
       </c>
       <c r="U55" t="s">
-        <v>264</v>
+        <v>301</v>
       </c>
       <c r="X55" t="s">
         <v>114</v>
       </c>
       <c r="Y55" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
     </row>
     <row r="56" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="B56" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="C56" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="D56" t="s">
         <v>72</v>
@@ -3606,13 +3606,13 @@
         <v>10.0877643</v>
       </c>
       <c r="M56" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T56" t="s">
-        <v>260</v>
+        <v>298</v>
       </c>
       <c r="U56" t="s">
-        <v>261</v>
+        <v>299</v>
       </c>
       <c r="X56" t="s">
         <v>114</v>
@@ -3626,13 +3626,13 @@
         <v>118</v>
       </c>
       <c r="B57" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="C57" t="s">
         <v>144</v>
       </c>
       <c r="D57" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="E57" t="s">
         <v>106</v>
@@ -3653,7 +3653,7 @@
         <v>0</v>
       </c>
       <c r="M57" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N57" t="s">
         <v>48</v>
@@ -3674,10 +3674,10 @@
         <v>1</v>
       </c>
       <c r="T57" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="U57" t="s">
-        <v>159</v>
+        <v>297</v>
       </c>
       <c r="X57" t="s">
         <v>114</v>
@@ -3691,13 +3691,13 @@
         <v>119</v>
       </c>
       <c r="B58" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="C58" t="s">
         <v>143</v>
       </c>
       <c r="D58" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="E58" t="s">
         <v>108</v>
@@ -3718,7 +3718,7 @@
         <v>0</v>
       </c>
       <c r="M58" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N58" t="s">
         <v>27</v>
@@ -3739,10 +3739,10 @@
         <v>1</v>
       </c>
       <c r="T58" t="s">
-        <v>308</v>
+        <v>285</v>
       </c>
       <c r="U58" t="s">
-        <v>309</v>
+        <v>286</v>
       </c>
       <c r="X58" t="s">
         <v>114</v>
@@ -3753,16 +3753,16 @@
     </row>
     <row r="59" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B59" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="C59" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D59" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="E59" t="s">
         <v>108</v>
@@ -3783,7 +3783,7 @@
         <v>0</v>
       </c>
       <c r="M59" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N59" t="s">
         <v>27</v>
@@ -3804,10 +3804,10 @@
         <v>1</v>
       </c>
       <c r="T59" t="s">
-        <v>310</v>
+        <v>295</v>
       </c>
       <c r="U59" t="s">
-        <v>311</v>
+        <v>296</v>
       </c>
       <c r="X59" t="s">
         <v>114</v>
@@ -3818,19 +3818,19 @@
     </row>
     <row r="60" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B60" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C60" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D60" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="E60" t="s">
-        <v>314</v>
+        <v>289</v>
       </c>
       <c r="F60" t="s">
         <v>135</v>
@@ -3848,13 +3848,13 @@
         <v>0</v>
       </c>
       <c r="M60" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N60" t="s">
         <v>48</v>
       </c>
       <c r="O60" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="P60" t="b">
         <v>1</v>
@@ -3869,10 +3869,10 @@
         <v>1</v>
       </c>
       <c r="T60" t="s">
-        <v>312</v>
+        <v>287</v>
       </c>
       <c r="U60" t="s">
-        <v>313</v>
+        <v>288</v>
       </c>
       <c r="X60" t="s">
         <v>114</v>
@@ -3883,19 +3883,19 @@
     </row>
     <row r="61" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="B61" t="s">
-        <v>265</v>
+        <v>249</v>
       </c>
       <c r="C61" t="s">
-        <v>266</v>
+        <v>250</v>
       </c>
       <c r="D61" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="E61" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="F61" t="s">
         <v>135</v>
@@ -3913,22 +3913,22 @@
         <v>0</v>
       </c>
       <c r="M61" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N61" t="s">
         <v>48</v>
       </c>
       <c r="O61" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="P61" t="b">
         <v>1</v>
       </c>
       <c r="T61" t="s">
-        <v>208</v>
+        <v>307</v>
       </c>
       <c r="U61" t="s">
-        <v>207</v>
+        <v>308</v>
       </c>
       <c r="X61" t="s">
         <v>114</v>
@@ -3939,19 +3939,19 @@
     </row>
     <row r="62" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B62" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C62" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D62" t="s">
         <v>24</v>
       </c>
       <c r="E62" t="s">
-        <v>272</v>
+        <v>256</v>
       </c>
       <c r="H62">
         <v>1855</v>
@@ -3969,30 +3969,30 @@
         <v>9.9354469999999999</v>
       </c>
       <c r="M62" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T62" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="U62" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="63" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B63" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="C63" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="D63" t="s">
         <v>72</v>
       </c>
       <c r="E63" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="F63" t="s">
         <v>135</v>
@@ -4016,13 +4016,13 @@
         <v>9.9354469999999999</v>
       </c>
       <c r="M63" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="T63" t="s">
-        <v>279</v>
+        <v>319</v>
       </c>
       <c r="U63" t="s">
-        <v>206</v>
+        <v>318</v>
       </c>
       <c r="X63" t="s">
         <v>114</v>
@@ -4033,16 +4033,16 @@
     </row>
     <row r="64" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="B64" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="C64" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="D64" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="E64" t="s">
         <v>106</v>
@@ -4063,10 +4063,10 @@
         <v>0</v>
       </c>
       <c r="M64" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N64" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="O64" t="s">
         <v>48</v>
@@ -4075,10 +4075,10 @@
         <v>1</v>
       </c>
       <c r="T64" t="s">
-        <v>280</v>
+        <v>262</v>
       </c>
       <c r="U64" t="s">
-        <v>281</v>
+        <v>263</v>
       </c>
       <c r="X64" t="s">
         <v>114</v>
@@ -4089,19 +4089,19 @@
     </row>
     <row r="65" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>286</v>
+        <v>268</v>
       </c>
       <c r="B65" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="C65" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="D65" t="s">
         <v>72</v>
       </c>
       <c r="E65" t="s">
-        <v>289</v>
+        <v>271</v>
       </c>
       <c r="F65" t="s">
         <v>135</v>
@@ -4125,7 +4125,7 @@
         <v>10.0877643</v>
       </c>
       <c r="M65" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="Q65" t="s">
         <v>135</v>
@@ -4137,10 +4137,10 @@
         <v>1</v>
       </c>
       <c r="T65" t="s">
-        <v>223</v>
+        <v>316</v>
       </c>
       <c r="U65" t="s">
-        <v>224</v>
+        <v>317</v>
       </c>
       <c r="X65" t="s">
         <v>114</v>
@@ -4151,19 +4151,19 @@
     </row>
     <row r="66" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>292</v>
+        <v>274</v>
       </c>
       <c r="B66" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
       <c r="C66" t="s">
-        <v>288</v>
+        <v>270</v>
       </c>
       <c r="D66" t="s">
         <v>72</v>
       </c>
       <c r="E66" t="s">
-        <v>289</v>
+        <v>271</v>
       </c>
       <c r="F66" t="s">
         <v>135</v>
@@ -4187,22 +4187,22 @@
         <v>10.0877643</v>
       </c>
       <c r="M66" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="Q66" t="s">
         <v>104</v>
       </c>
       <c r="R66" t="s">
-        <v>290</v>
+        <v>272</v>
       </c>
       <c r="S66" t="b">
         <v>1</v>
       </c>
       <c r="T66" t="s">
-        <v>293</v>
+        <v>314</v>
       </c>
       <c r="U66" t="s">
-        <v>294</v>
+        <v>315</v>
       </c>
       <c r="X66" t="s">
         <v>114</v>
@@ -4213,19 +4213,19 @@
     </row>
     <row r="67" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>298</v>
+        <v>278</v>
       </c>
       <c r="B67" t="s">
-        <v>296</v>
+        <v>276</v>
       </c>
       <c r="C67" t="s">
-        <v>297</v>
+        <v>277</v>
       </c>
       <c r="D67" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="E67" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="F67" t="s">
         <v>135</v>
@@ -4243,7 +4243,7 @@
         <v>0</v>
       </c>
       <c r="M67" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N67" t="s">
         <v>48</v>
@@ -4264,10 +4264,10 @@
         <v>1</v>
       </c>
       <c r="T67" t="s">
-        <v>299</v>
+        <v>313</v>
       </c>
       <c r="U67" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="X67" t="s">
         <v>114</v>
@@ -4278,19 +4278,19 @@
     </row>
     <row r="68" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>301</v>
+        <v>279</v>
       </c>
       <c r="B68" t="s">
-        <v>302</v>
+        <v>280</v>
       </c>
       <c r="C68" t="s">
-        <v>303</v>
+        <v>281</v>
       </c>
       <c r="D68" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="E68" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="F68" t="s">
         <v>135</v>
@@ -4308,31 +4308,31 @@
         <v>0</v>
       </c>
       <c r="M68" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N68" t="s">
         <v>48</v>
       </c>
       <c r="O68" t="s">
-        <v>284</v>
+        <v>266</v>
       </c>
       <c r="P68" t="b">
         <v>1</v>
       </c>
       <c r="Q68" t="s">
-        <v>290</v>
+        <v>272</v>
       </c>
       <c r="R68" t="s">
-        <v>284</v>
+        <v>266</v>
       </c>
       <c r="S68" t="b">
         <v>1</v>
       </c>
       <c r="T68" t="s">
-        <v>304</v>
+        <v>282</v>
       </c>
       <c r="U68" t="s">
-        <v>305</v>
+        <v>283</v>
       </c>
       <c r="X68" t="s">
         <v>114</v>
@@ -4343,13 +4343,13 @@
     </row>
     <row r="69" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B69" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C69" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D69" t="s">
         <v>72</v>
@@ -4373,21 +4373,21 @@
         <v>11.00703</v>
       </c>
       <c r="M69" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="T69" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="70" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>191</v>
+      </c>
+      <c r="B70" t="s">
+        <v>192</v>
+      </c>
+      <c r="C70" t="s">
         <v>195</v>
-      </c>
-      <c r="B70" t="s">
-        <v>196</v>
-      </c>
-      <c r="C70" t="s">
-        <v>199</v>
       </c>
       <c r="D70" t="s">
         <v>72</v>
@@ -4411,18 +4411,18 @@
         <v>9.08</v>
       </c>
       <c r="M70" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="71" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B71" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C71" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="D71" t="s">
         <v>72</v>
@@ -4446,7 +4446,7 @@
         <v>8.2777499999999993</v>
       </c>
       <c r="M71" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>